<commit_message>
Reconcile six TPBank evidence descriptions with period reports
</commit_message>
<xml_diff>
--- a/Code/CleanData.xlsx
+++ b/Code/CleanData.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh_muc" sheetId="1" r:id="R8badd14026644e83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TPBank" sheetId="2" r:id="Re3f131cdfa8d4cde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDBank" sheetId="3" r:id="Re16bc6090cf24def"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LP Bank" sheetId="4" r:id="R942f149d9179462e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OCB" sheetId="5" r:id="Ra3f3e2b4a75249f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SaigonBank" sheetId="6" r:id="Rb7daab92b32e426b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong_hop" sheetId="7" r:id="Rf009597b7fcb46dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loi_can_ra_soat" sheetId="8" r:id="Rf464525e1dc2468a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh_muc" sheetId="1" r:id="Rc7239fd9103a4f5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TPBank" sheetId="2" r:id="Raad20a876cc041e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDBank" sheetId="3" r:id="R414586961e024eae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LP Bank" sheetId="4" r:id="R6643f3791b604619"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OCB" sheetId="5" r:id="Rc4ce16a8c4fe43f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SaigonBank" sheetId="6" r:id="Rdc3a6378fe2d48be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong_hop" sheetId="7" r:id="R8cd1836bc2ab4ed0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loi_can_ra_soat" sheetId="8" r:id="R16740cb4bbcd4915"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10072,12 +10072,9 @@
         <ns0:v>2</ns0:v>
       </ns0:c>
       <ns0:c r="F50" t="str">
-        <ns0:v>TPBank công bố tiếp nhận hàng nghìn đề xuất/sáng kiến và triển khai các sáng kiến vào nghiệp vụ, quy trình, sản phẩm. Điều này phù hợp việc nhận diện, khuyến khích áp dụng thông lệ/sáng kiến tại một số bộ phận; chưa đủ xác nhận toàn bộ ngân hàng. TPBank
+        <ns0:v>Báo cáo PTBV 2024 ghi nhận TPBank hoàn thành 238 yêu cầu cải tiến cho các đơn vị trong hệ thống và số hóa 523 quy trình. Nội dung thể hiện việc triển khai các cải tiến vào hoạt động; tài liệu này không mô tả quy trình tổng kết và nhân rộng bài học thành công trên toàn ngân hàng.
 Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 60
-https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=60
-Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 79
-https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=79
-Phạm vi nguồn bổ sung: Nguồn 2024 xác nhận 238 yêu cầu cải tiến và cơ chế thưởng sáng kiến. Con số hàng nghìn đề xuất tìm được trong bài công bố 2022 nói về năm 2021, chưa xác định được nguồn cho con số này trong kỳ 2023–2025.</ns0:v>
+https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=60</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="51">
@@ -10185,14 +10182,13 @@
         <ns0:v>4</ns0:v>
       </ns0:c>
       <ns0:c r="F55" t="str">
-        <ns0:v>TPBank chủ động ứng dụng AI, Big Data, Machine Learning, sinh trắc học, Cloud, Active-Active DC-DR, SD-WAN và OpenAPI vào hoạt động. Đây là bằng chứng ngân hàng chủ động tìm kiếm và ứng dụng công nghệ mới; chưa chứng minh việc này mở rộng cùng toàn bộ đối tác hệ sinh thái. TPBank
+        <ns0:v>Trong giai đoạn 2023–2025, TPBank công bố ứng dụng AI, Big Data, Machine Learning, Bio Center và Open API; eBankX/eBankBiz vận hành trên container, tự co giãn và nền tảng Microservice/Cloud. Năm 2025, ngân hàng tiếp tục nâng cấp ESB cloud ready và chuyển đổi dịch vụ Microservice. Các nguồn này mô tả việc chủ động triển khai công nghệ trong hoạt động ngân hàng, không xác định mức triển khai của toàn bộ đối tác hệ sinh thái.
+Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 59
+https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=59
 Nguồn: Báo cáo thường niên TPBank 2023 · trang PDF 26 (trang in 48–49)
 https://static2.vietstock.vn/data/HOSE/2023/BCTN/VN/TPB_Baocaothuongnien_2023/maket+n%E1%BB%9Bi+x%C3%A9n+2024+-+view+15.4.2024+RESIZE.pdf#page=26
 Nguồn: Báo cáo thường niên TPBank 2025 · trang PDF 24 (trang in 44–45)
-https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/TPB_Baocaothuongnien_2025/BCTN+2026+TV+20.4+VIEW-2.pdf#page=24
-Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 59
-https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=59
-Phạm vi nguồn bổ sung: Nguồn trong kỳ xác nhận Cloud, nền tảng số và vận hành liên tục. Các chi tiết Active-Active DC-DR và SD-WAN tìm được trong bài công bố 2022; chưa tìm thấy xác nhận lại cấu hình đó trong tài liệu 2023–2025 đã đọc.</ns0:v>
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/TPB_Baocaothuongnien_2025/BCTN+2026+TV+20.4+VIEW-2.pdf#page=24</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="56">
@@ -10340,14 +10336,11 @@
         <ns0:v>3</ns0:v>
       </ns0:c>
       <ns0:c r="F62" t="str">
-        <ns0:v>Hạ tầng Active-Active DC-DR, Cloud, SD-WAN và các nền tảng ngân hàng số cho thấy kiến trúc công nghệ hỗ trợ triển khai nhiều ứng dụng quan trọng; chưa đủ xác nhận triển khai liền mạch mọi ứng dụng. TPBank
+        <ns0:v>BCTN 2023 cho biết eBankX và eBankBiz hoạt động hoàn toàn trên nền tảng container, auto scale và ứng dụng Microservice/Cloud platform. BCTN 2025 ghi nhận nâng cấp ESB lên ACE cloud ready, nâng cấp Open API và chuyển đổi dịch vụ Microservice. Nội dung mô tả kiến trúc hỗ trợ các nền tảng ngân hàng số; chưa mô tả sự tích hợp liền mạch của mọi ứng dụng.
 Nguồn: Báo cáo thường niên TPBank 2023 · trang PDF 26 (trang in 48–49)
 https://static2.vietstock.vn/data/HOSE/2023/BCTN/VN/TPB_Baocaothuongnien_2023/maket+n%E1%BB%9Bi+x%C3%A9n+2024+-+view+15.4.2024+RESIZE.pdf#page=26
 Nguồn: Báo cáo thường niên TPBank 2025 · trang PDF 24 (trang in 44–45)
-https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/TPB_Baocaothuongnien_2025/BCTN+2026+TV+20.4+VIEW-2.pdf#page=24
-Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 59
-https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=59
-Phạm vi nguồn bổ sung: Nguồn trong kỳ xác nhận Cloud, nền tảng số và vận hành liên tục. Các chi tiết Active-Active DC-DR và SD-WAN tìm được trong bài công bố 2022; chưa tìm thấy xác nhận lại cấu hình đó trong tài liệu 2023–2025 đã đọc.</ns0:v>
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/TPB_Baocaothuongnien_2025/BCTN+2026+TV+20.4+VIEW-2.pdf#page=24</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="63">
@@ -10623,14 +10616,11 @@
         <ns0:v>3</ns0:v>
       </ns0:c>
       <ns0:c r="F75" t="str">
-        <ns0:v>TPBank có hạ tầng Active-Active DC-DR, Cloud, SD-WAN và LiveBank; điều này cho thấy quản lý hạ tầng đáp ứng phần lớn nhu cầu vận hành, nhưng chưa có dữ liệu về tích hợp/cải tiến liên tục toàn diện. TPBank
-Nguồn: Báo cáo thường niên TPBank 2023 · trang PDF 26 (trang in 48–49)
-https://static2.vietstock.vn/data/HOSE/2023/BCTN/VN/TPB_Baocaothuongnien_2023/maket+n%E1%BB%9Bi+x%C3%A9n+2024+-+view+15.4.2024+RESIZE.pdf#page=26
+        <ns0:v>BCTN 2025 ghi nhận mở rộng máy chủ vật lý, máy chủ ảo private cloud, lưu trữ, đường truyền và cơ sở dữ liệu để đáp ứng nhu cầu vận hành và phát triển. Ngân hàng triển khai cập nhật core banking không dừng, nâng cấp ESB cloud ready và chuyển đổi dịch vụ Microservice. Các nội dung thể hiện việc quản lý và nâng cấp hạ tầng phục vụ hoạt động ngân hàng.
 Nguồn: Báo cáo thường niên TPBank 2025 · trang PDF 24 (trang in 44–45)
 https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/TPB_Baocaothuongnien_2025/BCTN+2026+TV+20.4+VIEW-2.pdf#page=24
 Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 59
-https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=59
-Phạm vi nguồn bổ sung: Nguồn trong kỳ xác nhận Cloud, nền tảng số và vận hành liên tục. Các chi tiết Active-Active DC-DR và SD-WAN tìm được trong bài công bố 2022; chưa tìm thấy xác nhận lại cấu hình đó trong tài liệu 2023–2025 đã đọc.</ns0:v>
+https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=59</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="76">
@@ -11042,14 +11032,13 @@
         <ns0:v>3</ns0:v>
       </ns0:c>
       <ns0:c r="F94" t="str">
-        <ns0:v>TPBank vận hành LiveBank 24/7, nền tảng số có tỷ lệ giao dịch rất cao và hệ thống dự phòng Active-Active DC-DR. Bằng chứng thể hiện năng lực duy trì dịch vụ, nhưng không có SLA công khai để xác nhận Mức 4. TPBank
-Nguồn: Báo cáo thường niên TPBank 2023 · trang PDF 26 (trang in 48–49)
-https://static2.vietstock.vn/data/HOSE/2023/BCTN/VN/TPB_Baocaothuongnien_2023/maket+n%E1%BB%9Bi+x%C3%A9n+2024+-+view+15.4.2024+RESIZE.pdf#page=26
-Nguồn: Báo cáo thường niên TPBank 2025 · trang PDF 24 (trang in 44–45)
-https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/TPB_Baocaothuongnien_2025/BCTN+2026+TV+20.4+VIEW-2.pdf#page=24
+        <ns0:v>Báo cáo PTBV 2024 ghi nhận LiveBank 24/7, nâng cấp core banking không cần tạm dừng giao dịch và chứng chỉ ISO 22301 về quản lý kinh doanh liên tục. BCTN 2025 ghi nhận cập nhật core banking không dừng; thời gian gián đoạn dịch vụ giảm 40%, thời gian dừng chủ động giảm 20% và từ tháng 02/2025 không phát sinh sự cố dừng eBank. Đây là kết quả công bố theo từng nguồn, không phải cam kết SLA cho toàn bộ dịch vụ.
 Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 59
 https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=59
-Phạm vi nguồn bổ sung: Nguồn trong kỳ xác nhận Cloud, nền tảng số và vận hành liên tục. Các chi tiết Active-Active DC-DR và SD-WAN tìm được trong bài công bố 2022; chưa tìm thấy xác nhận lại cấu hình đó trong tài liệu 2023–2025 đã đọc.</ns0:v>
+Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 61
+https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=61
+Nguồn: Báo cáo thường niên TPBank 2025 · trang PDF 24 (trang in 44–45)
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/TPB_Baocaothuongnien_2025/BCTN+2026+TV+20.4+VIEW-2.pdf#page=24</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="95">
@@ -11533,12 +11522,11 @@
         <ns0:v>2</ns0:v>
       </ns0:c>
       <ns0:c r="F117" t="str">
-        <ns0:v>TPBank tiếp nhận hàng nghìn sáng kiến trong nghiệp vụ, quy trình, sản phẩm và dịch vụ, cho thấy tồn tại môi trường khuyến khích đổi mới; chưa có bằng chứng áp dụng tại hầu hết/toàn bộ đơn vị. TPBank
-Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 60
-https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=60
+        <ns0:v>Báo cáo PTBV 2024 mô tả cơ chế thưởng đột xuất cho cá nhân hoặc tập thể có sáng kiến cải tiến kỹ thuật, quy trình nghiệp vụ mang lại hiệu quả. Cùng năm, TPBank hoàn thành 238 yêu cầu cải tiến cho các đơn vị trong hệ thống. Đây là hoạt động khuyến khích và triển khai đổi mới; số liệu không đo mức độ tham gia của từng đơn vị.
 Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 79
 https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=79
-Phạm vi nguồn bổ sung: Nguồn 2024 xác nhận 238 yêu cầu cải tiến và cơ chế thưởng sáng kiến. Con số hàng nghìn đề xuất tìm được trong bài công bố 2022 nói về năm 2021, chưa xác định được nguồn cho con số này trong kỳ 2023–2025.</ns0:v>
+Nguồn: Báo cáo phát triển bền vững TPBank 2024 · trang PDF 60
+https://tpb.vn/wps/wcm/connect/36035be7-468c-459e-a586-fc20f694f0c0/2025.11.03+TPBank+_+B%C3%A1o+c%C3%A1o+ph%C3%A1t+tri%E1%BB%83n+b%E1%BB%81n+v%E1%BB%AFng+n%C4%83m+2024+BOD+ph%C3%AA+duy%E1%BB%87t.pdf?MOD=AJPERES&amp;CONVERT_TO=url&amp;CACHEID=ROOTWORKSPACE-36035be7-468c-459e-a586-fc20f694f0c0-pFhGccW#page=60</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="118">

</xml_diff>

<commit_message>
Remove obsolete review labels from approved workbooks and dashboard
</commit_message>
<xml_diff>
--- a/Code/CleanData.xlsx
+++ b/Code/CleanData.xlsx
@@ -1,17 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh_muc" sheetId="1" r:id="Rc7239fd9103a4f5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TPBank" sheetId="2" r:id="Raad20a876cc041e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDBank" sheetId="3" r:id="R414586961e024eae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LP Bank" sheetId="4" r:id="R6643f3791b604619"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OCB" sheetId="5" r:id="Rc4ce16a8c4fe43f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SaigonBank" sheetId="6" r:id="Rdc3a6378fe2d48be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong_hop" sheetId="7" r:id="R8cd1836bc2ab4ed0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loi_can_ra_soat" sheetId="8" r:id="R16740cb4bbcd4915"/>
-  </x:sheets>
-</x:workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:sheets>
+    <ns0:sheet name="Danh_muc" sheetId="1" ns1:id="R8d0f85caf8ac45a1"/>
+    <ns0:sheet name="TPBank" sheetId="2" ns1:id="Rdbc1d0adb1424f4a"/>
+    <ns0:sheet name="HDBank" sheetId="3" ns1:id="Rc280ebc6d5cb492c"/>
+    <ns0:sheet name="LP Bank" sheetId="4" ns1:id="R44643caaa547486c"/>
+    <ns0:sheet name="OCB" sheetId="5" ns1:id="R1fee4504302141d0"/>
+    <ns0:sheet name="SaigonBank" sheetId="6" ns1:id="R1bc343f07fa34c46"/>
+    <ns0:sheet name="Tong_hop" sheetId="7" ns1:id="Rafd86e17680e49bb"/>
+  </ns0:sheets>
+</ns0:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4516,39 +4515,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">SaigonBank</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sheet</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Loại lỗi</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Chi tiết</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Trạng thái</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Rà soát mức 0</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Xác nhận đã rà soát nguồn và thực sự không có thông tin công bố.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cần rà soát</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Toàn bộ dữ liệu</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Chưa kiểm tra được năm tự động</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Các sheet ngân hàng chưa có cột Năm riêng. Cần xác nhận bằng chứng thuộc năm 2023, 2024 hay 2025 trước khi phân tích theo năm.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cần bổ sung cấu trúc</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -23600,1565 +23566,4 @@
   <ns0:autoFilter ref="A1:G6" ns1:uid="{00000000-0009-0000-0000-000006000000}"/>
   <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </ns0:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
-  <ns0:sheetFormatPr defaultRowHeight="14.5"/>
-  <ns0:cols>
-    <ns0:col min="1" max="1" width="17" customWidth="1"/>
-    <ns0:col min="2" max="2" width="12" customWidth="1"/>
-    <ns0:col min="3" max="3" width="32" customWidth="1"/>
-    <ns0:col min="4" max="4" width="55" customWidth="1"/>
-    <ns0:col min="5" max="5" width="22" customWidth="1"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1">
-      <ns0:c r="A1" s="1" t="s">
-        <ns0:v>1499</ns0:v>
-      </ns0:c>
-      <ns0:c r="B1" s="1" t="s">
-        <ns0:v>2</ns0:v>
-      </ns0:c>
-      <ns0:c r="C1" s="1" t="s">
-        <ns0:v>1500</ns0:v>
-      </ns0:c>
-      <ns0:c r="D1" s="1" t="s">
-        <ns0:v>1501</ns0:v>
-      </ns0:c>
-      <ns0:c r="E1" s="1" t="s">
-        <ns0:v>1502</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="2">
-      <ns0:c r="A2" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B2" t="s">
-        <ns0:v>39</ns0:v>
-      </ns0:c>
-      <ns0:c r="C2" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D2" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E2" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="3">
-      <ns0:c r="A3" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B3" t="s">
-        <ns0:v>60</ns0:v>
-      </ns0:c>
-      <ns0:c r="C3" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D3" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E3" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="4">
-      <ns0:c r="A4" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B4" t="s">
-        <ns0:v>75</ns0:v>
-      </ns0:c>
-      <ns0:c r="C4" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D4" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E4" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5">
-      <ns0:c r="A5" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B5" t="s">
-        <ns0:v>89</ns0:v>
-      </ns0:c>
-      <ns0:c r="C5" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D5" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E5" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="6">
-      <ns0:c r="A6" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B6" t="s">
-        <ns0:v>110</ns0:v>
-      </ns0:c>
-      <ns0:c r="C6" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D6" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E6" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="7">
-      <ns0:c r="A7" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B7" t="s">
-        <ns0:v>124</ns0:v>
-      </ns0:c>
-      <ns0:c r="C7" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D7" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E7" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="8">
-      <ns0:c r="A8" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B8" t="s">
-        <ns0:v>132</ns0:v>
-      </ns0:c>
-      <ns0:c r="C8" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D8" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E8" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="9">
-      <ns0:c r="A9" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B9" t="s">
-        <ns0:v>139</ns0:v>
-      </ns0:c>
-      <ns0:c r="C9" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D9" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E9" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="10">
-      <ns0:c r="A10" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B10" t="s">
-        <ns0:v>154</ns0:v>
-      </ns0:c>
-      <ns0:c r="C10" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D10" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E10" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="11">
-      <ns0:c r="A11" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B11" t="s">
-        <ns0:v>161</ns0:v>
-      </ns0:c>
-      <ns0:c r="C11" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D11" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E11" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="12">
-      <ns0:c r="A12" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B12" t="s">
-        <ns0:v>182</ns0:v>
-      </ns0:c>
-      <ns0:c r="C12" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D12" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E12" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="13">
-      <ns0:c r="A13" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B13" t="s">
-        <ns0:v>191</ns0:v>
-      </ns0:c>
-      <ns0:c r="C13" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D13" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E13" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="14">
-      <ns0:c r="A14" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B14" t="s">
-        <ns0:v>198</ns0:v>
-      </ns0:c>
-      <ns0:c r="C14" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D14" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E14" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="15">
-      <ns0:c r="A15" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B15" t="s">
-        <ns0:v>205</ns0:v>
-      </ns0:c>
-      <ns0:c r="C15" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D15" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E15" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="16">
-      <ns0:c r="A16" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B16" t="s">
-        <ns0:v>212</ns0:v>
-      </ns0:c>
-      <ns0:c r="C16" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D16" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E16" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="17">
-      <ns0:c r="A17" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B17" t="s">
-        <ns0:v>242</ns0:v>
-      </ns0:c>
-      <ns0:c r="C17" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D17" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E17" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="18">
-      <ns0:c r="A18" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B18" t="s">
-        <ns0:v>249</ns0:v>
-      </ns0:c>
-      <ns0:c r="C18" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D18" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E18" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="19">
-      <ns0:c r="A19" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B19" t="s">
-        <ns0:v>256</ns0:v>
-      </ns0:c>
-      <ns0:c r="C19" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D19" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E19" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="20">
-      <ns0:c r="A20" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B20" t="s">
-        <ns0:v>264</ns0:v>
-      </ns0:c>
-      <ns0:c r="C20" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D20" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E20" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="21">
-      <ns0:c r="A21" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B21" t="s">
-        <ns0:v>278</ns0:v>
-      </ns0:c>
-      <ns0:c r="C21" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D21" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E21" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="22">
-      <ns0:c r="A22" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B22" t="s">
-        <ns0:v>315</ns0:v>
-      </ns0:c>
-      <ns0:c r="C22" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D22" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E22" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="23">
-      <ns0:c r="A23" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B23" t="s">
-        <ns0:v>380</ns0:v>
-      </ns0:c>
-      <ns0:c r="C23" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D23" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E23" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="24">
-      <ns0:c r="A24" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B24" t="s">
-        <ns0:v>387</ns0:v>
-      </ns0:c>
-      <ns0:c r="C24" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D24" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E24" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="25">
-      <ns0:c r="A25" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B25" t="s">
-        <ns0:v>409</ns0:v>
-      </ns0:c>
-      <ns0:c r="C25" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D25" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E25" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="26">
-      <ns0:c r="A26" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B26" t="s">
-        <ns0:v>416</ns0:v>
-      </ns0:c>
-      <ns0:c r="C26" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D26" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E26" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="27">
-      <ns0:c r="A27" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B27" t="s">
-        <ns0:v>423</ns0:v>
-      </ns0:c>
-      <ns0:c r="C27" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D27" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E27" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="28">
-      <ns0:c r="A28" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B28" t="s">
-        <ns0:v>452</ns0:v>
-      </ns0:c>
-      <ns0:c r="C28" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D28" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E28" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="29">
-      <ns0:c r="A29" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B29" t="s">
-        <ns0:v>459</ns0:v>
-      </ns0:c>
-      <ns0:c r="C29" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D29" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E29" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="30">
-      <ns0:c r="A30" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B30" t="s">
-        <ns0:v>473</ns0:v>
-      </ns0:c>
-      <ns0:c r="C30" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D30" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E30" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="31">
-      <ns0:c r="A31" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B31" t="s">
-        <ns0:v>495</ns0:v>
-      </ns0:c>
-      <ns0:c r="C31" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D31" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E31" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="32">
-      <ns0:c r="A32" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B32" t="s">
-        <ns0:v>502</ns0:v>
-      </ns0:c>
-      <ns0:c r="C32" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D32" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E32" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="33">
-      <ns0:c r="A33" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B33" t="s">
-        <ns0:v>510</ns0:v>
-      </ns0:c>
-      <ns0:c r="C33" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D33" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E33" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="34">
-      <ns0:c r="A34" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B34" t="s">
-        <ns0:v>517</ns0:v>
-      </ns0:c>
-      <ns0:c r="C34" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D34" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E34" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="35">
-      <ns0:c r="A35" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B35" t="s">
-        <ns0:v>524</ns0:v>
-      </ns0:c>
-      <ns0:c r="C35" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D35" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E35" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="36">
-      <ns0:c r="A36" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B36" t="s">
-        <ns0:v>545</ns0:v>
-      </ns0:c>
-      <ns0:c r="C36" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D36" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E36" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="37">
-      <ns0:c r="A37" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B37" t="s">
-        <ns0:v>559</ns0:v>
-      </ns0:c>
-      <ns0:c r="C37" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D37" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E37" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="38">
-      <ns0:c r="A38" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B38" t="s">
-        <ns0:v>596</ns0:v>
-      </ns0:c>
-      <ns0:c r="C38" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D38" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E38" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="39">
-      <ns0:c r="A39" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B39" t="s">
-        <ns0:v>604</ns0:v>
-      </ns0:c>
-      <ns0:c r="C39" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D39" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E39" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="40">
-      <ns0:c r="A40" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B40" t="s">
-        <ns0:v>611</ns0:v>
-      </ns0:c>
-      <ns0:c r="C40" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D40" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E40" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="41">
-      <ns0:c r="A41" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B41" t="s">
-        <ns0:v>618</ns0:v>
-      </ns0:c>
-      <ns0:c r="C41" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D41" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E41" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="42">
-      <ns0:c r="A42" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B42" t="s">
-        <ns0:v>647</ns0:v>
-      </ns0:c>
-      <ns0:c r="C42" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D42" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E42" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="43">
-      <ns0:c r="A43" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B43" t="s">
-        <ns0:v>654</ns0:v>
-      </ns0:c>
-      <ns0:c r="C43" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D43" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E43" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="44">
-      <ns0:c r="A44" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B44" t="s">
-        <ns0:v>661</ns0:v>
-      </ns0:c>
-      <ns0:c r="C44" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D44" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E44" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="45">
-      <ns0:c r="A45" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B45" t="s">
-        <ns0:v>668</ns0:v>
-      </ns0:c>
-      <ns0:c r="C45" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D45" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E45" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="46">
-      <ns0:c r="A46" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B46" t="s">
-        <ns0:v>683</ns0:v>
-      </ns0:c>
-      <ns0:c r="C46" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D46" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E46" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="47">
-      <ns0:c r="A47" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B47" t="s">
-        <ns0:v>690</ns0:v>
-      </ns0:c>
-      <ns0:c r="C47" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D47" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E47" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="48">
-      <ns0:c r="A48" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B48" t="s">
-        <ns0:v>704</ns0:v>
-      </ns0:c>
-      <ns0:c r="C48" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D48" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E48" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="49">
-      <ns0:c r="A49" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B49" t="s">
-        <ns0:v>711</ns0:v>
-      </ns0:c>
-      <ns0:c r="C49" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D49" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E49" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="50">
-      <ns0:c r="A50" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B50" t="s">
-        <ns0:v>741</ns0:v>
-      </ns0:c>
-      <ns0:c r="C50" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D50" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E50" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="51">
-      <ns0:c r="A51" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B51" t="s">
-        <ns0:v>755</ns0:v>
-      </ns0:c>
-      <ns0:c r="C51" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D51" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E51" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="52">
-      <ns0:c r="A52" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B52" t="s">
-        <ns0:v>762</ns0:v>
-      </ns0:c>
-      <ns0:c r="C52" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D52" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E52" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="53">
-      <ns0:c r="A53" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B53" t="s">
-        <ns0:v>769</ns0:v>
-      </ns0:c>
-      <ns0:c r="C53" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D53" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E53" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="54">
-      <ns0:c r="A54" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B54" t="s">
-        <ns0:v>777</ns0:v>
-      </ns0:c>
-      <ns0:c r="C54" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D54" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E54" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="55">
-      <ns0:c r="A55" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B55" t="s">
-        <ns0:v>784</ns0:v>
-      </ns0:c>
-      <ns0:c r="C55" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D55" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E55" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="56">
-      <ns0:c r="A56" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B56" t="s">
-        <ns0:v>791</ns0:v>
-      </ns0:c>
-      <ns0:c r="C56" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D56" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E56" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="57">
-      <ns0:c r="A57" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B57" t="s">
-        <ns0:v>798</ns0:v>
-      </ns0:c>
-      <ns0:c r="C57" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D57" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E57" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="58">
-      <ns0:c r="A58" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B58" t="s">
-        <ns0:v>805</ns0:v>
-      </ns0:c>
-      <ns0:c r="C58" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D58" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E58" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="59">
-      <ns0:c r="A59" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B59" t="s">
-        <ns0:v>819</ns0:v>
-      </ns0:c>
-      <ns0:c r="C59" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D59" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E59" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="60">
-      <ns0:c r="A60" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B60" t="s">
-        <ns0:v>826</ns0:v>
-      </ns0:c>
-      <ns0:c r="C60" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D60" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E60" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="61">
-      <ns0:c r="A61" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B61" t="s">
-        <ns0:v>855</ns0:v>
-      </ns0:c>
-      <ns0:c r="C61" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D61" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E61" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="62">
-      <ns0:c r="A62" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B62" t="s">
-        <ns0:v>862</ns0:v>
-      </ns0:c>
-      <ns0:c r="C62" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D62" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E62" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="63">
-      <ns0:c r="A63" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B63" t="s">
-        <ns0:v>869</ns0:v>
-      </ns0:c>
-      <ns0:c r="C63" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D63" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E63" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="64">
-      <ns0:c r="A64" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B64" t="s">
-        <ns0:v>876</ns0:v>
-      </ns0:c>
-      <ns0:c r="C64" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D64" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E64" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="65">
-      <ns0:c r="A65" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B65" t="s">
-        <ns0:v>883</ns0:v>
-      </ns0:c>
-      <ns0:c r="C65" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D65" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E65" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="66">
-      <ns0:c r="A66" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B66" t="s">
-        <ns0:v>892</ns0:v>
-      </ns0:c>
-      <ns0:c r="C66" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D66" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E66" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="67">
-      <ns0:c r="A67" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B67" t="s">
-        <ns0:v>899</ns0:v>
-      </ns0:c>
-      <ns0:c r="C67" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D67" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E67" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="68">
-      <ns0:c r="A68" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B68" t="s">
-        <ns0:v>906</ns0:v>
-      </ns0:c>
-      <ns0:c r="C68" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D68" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E68" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="69">
-      <ns0:c r="A69" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B69" t="s">
-        <ns0:v>927</ns0:v>
-      </ns0:c>
-      <ns0:c r="C69" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D69" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E69" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="70">
-      <ns0:c r="A70" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B70" t="s">
-        <ns0:v>934</ns0:v>
-      </ns0:c>
-      <ns0:c r="C70" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D70" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E70" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="71">
-      <ns0:c r="A71" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B71" t="s">
-        <ns0:v>949</ns0:v>
-      </ns0:c>
-      <ns0:c r="C71" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D71" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E71" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="72">
-      <ns0:c r="A72" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B72" t="s">
-        <ns0:v>956</ns0:v>
-      </ns0:c>
-      <ns0:c r="C72" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D72" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E72" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="73">
-      <ns0:c r="A73" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B73" t="s">
-        <ns0:v>963</ns0:v>
-      </ns0:c>
-      <ns0:c r="C73" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D73" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E73" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="74">
-      <ns0:c r="A74" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B74" t="s">
-        <ns0:v>970</ns0:v>
-      </ns0:c>
-      <ns0:c r="C74" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D74" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E74" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="75">
-      <ns0:c r="A75" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B75" t="s">
-        <ns0:v>984</ns0:v>
-      </ns0:c>
-      <ns0:c r="C75" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D75" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E75" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="76">
-      <ns0:c r="A76" t="s">
-        <ns0:v>1494</ns0:v>
-      </ns0:c>
-      <ns0:c r="B76" t="s">
-        <ns0:v>991</ns0:v>
-      </ns0:c>
-      <ns0:c r="C76" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D76" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E76" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="77">
-      <ns0:c r="A77" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B77" t="s">
-        <ns0:v>39</ns0:v>
-      </ns0:c>
-      <ns0:c r="C77" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D77" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E77" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="78">
-      <ns0:c r="A78" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B78" t="s">
-        <ns0:v>60</ns0:v>
-      </ns0:c>
-      <ns0:c r="C78" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D78" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E78" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="79">
-      <ns0:c r="A79" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B79" t="s">
-        <ns0:v>249</ns0:v>
-      </ns0:c>
-      <ns0:c r="C79" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D79" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E79" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="80">
-      <ns0:c r="A80" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B80" t="s">
-        <ns0:v>357</ns0:v>
-      </ns0:c>
-      <ns0:c r="C80" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D80" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E80" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="81">
-      <ns0:c r="A81" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B81" t="s">
-        <ns0:v>416</ns0:v>
-      </ns0:c>
-      <ns0:c r="C81" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D81" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E81" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="82">
-      <ns0:c r="A82" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B82" t="s">
-        <ns0:v>531</ns0:v>
-      </ns0:c>
-      <ns0:c r="C82" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D82" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E82" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="83">
-      <ns0:c r="A83" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B83" t="s">
-        <ns0:v>596</ns0:v>
-      </ns0:c>
-      <ns0:c r="C83" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D83" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E83" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="84">
-      <ns0:c r="A84" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B84" t="s">
-        <ns0:v>611</ns0:v>
-      </ns0:c>
-      <ns0:c r="C84" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D84" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E84" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="85">
-      <ns0:c r="A85" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B85" t="s">
-        <ns0:v>668</ns0:v>
-      </ns0:c>
-      <ns0:c r="C85" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D85" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E85" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="86">
-      <ns0:c r="A86" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B86" t="s">
-        <ns0:v>755</ns0:v>
-      </ns0:c>
-      <ns0:c r="C86" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D86" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E86" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="87">
-      <ns0:c r="A87" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B87" t="s">
-        <ns0:v>762</ns0:v>
-      </ns0:c>
-      <ns0:c r="C87" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D87" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E87" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="88">
-      <ns0:c r="A88" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B88" t="s">
-        <ns0:v>892</ns0:v>
-      </ns0:c>
-      <ns0:c r="C88" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D88" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E88" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="89">
-      <ns0:c r="A89" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B89" t="s">
-        <ns0:v>906</ns0:v>
-      </ns0:c>
-      <ns0:c r="C89" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D89" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E89" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="90">
-      <ns0:c r="A90" t="s">
-        <ns0:v>1497</ns0:v>
-      </ns0:c>
-      <ns0:c r="B90" t="s">
-        <ns0:v>970</ns0:v>
-      </ns0:c>
-      <ns0:c r="C90" t="s">
-        <ns0:v>1503</ns0:v>
-      </ns0:c>
-      <ns0:c r="D90" t="s">
-        <ns0:v>1504</ns0:v>
-      </ns0:c>
-      <ns0:c r="E90" t="s">
-        <ns0:v>1505</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="91">
-      <ns0:c r="A91" t="s">
-        <ns0:v>1506</ns0:v>
-      </ns0:c>
-      <ns0:c r="C91" t="s">
-        <ns0:v>1507</ns0:v>
-      </ns0:c>
-      <ns0:c r="D91" t="s">
-        <ns0:v>1508</ns0:v>
-      </ns0:c>
-      <ns0:c r="E91" t="s">
-        <ns0:v>1509</ns0:v>
-      </ns0:c>
-    </ns0:row>
-  </ns0:sheetData>
-  <ns0:autoFilter ref="A1:E91" ns1:uid="{00000000-0009-0000-0000-000007000000}"/>
-  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</ns0:worksheet>
 </file>
</xml_diff>

<commit_message>
Update LPBank and Saigonbank citations within 2023-2025
</commit_message>
<xml_diff>
--- a/Code/CleanData.xlsx
+++ b/Code/CleanData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="Danh_muc" sheetId="1" r:id="R8d0f85caf8ac45a1"/>
-    <sheet name="TPBank" sheetId="2" r:id="Rdbc1d0adb1424f4a"/>
-    <sheet name="HDBank" sheetId="3" r:id="Rc280ebc6d5cb492c"/>
-    <sheet name="LP Bank" sheetId="4" r:id="R44643caaa547486c"/>
-    <sheet name="OCB" sheetId="5" r:id="R1fee4504302141d0"/>
-    <sheet name="SaigonBank" sheetId="6" r:id="R1bc343f07fa34c46"/>
-    <sheet name="Tong_hop" sheetId="7" r:id="Rafd86e17680e49bb"/>
-  </sheets>
-</workbook>
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh_muc" sheetId="1" r:id="R7736cafa2a104168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TPBank" sheetId="2" r:id="R52b126d43a9c4add"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDBank" sheetId="3" r:id="Re15cde1358304955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LP Bank" sheetId="4" r:id="R846d4f46dcc74373"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OCB" sheetId="5" r:id="R08646ca547c9445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SaigonBank" sheetId="6" r:id="Rb61bc0d15e1644c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong_hop" sheetId="7" r:id="R3f4cf67300424cc2"/>
+  </x:sheets>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3361,15 +3361,9 @@
     <x:t xml:space="preserve">S</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Triển khai các tính năng cá nhân hóa dịch vụ ở một số khía cạnh như giao diện cá nhân hóa trên LPBank Plus, đặt tên tài khoản iName, chọn số tài khoản đẹp, giao diện riêng cho phân khúc khách hàng LPBank Priority. Tuy nhiên, chưa có số liệu đo lường định lượng về tỷ lệ khách hàng thực tế sử dụng tính năng cá nhân hóa. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Có một số gói sản phẩm và thông điệp tiếp thị hướng đến từng phân khúc khách hàng mục tiêu riêng biệt (hộ kinh doanh Lộc Phát Pay, hưu trí, lực lượng vũ trang, an sinh xã hội). Báo cáo chưa công bố chỉ số đo lường hiệu quả chuyển đổi hay tỷ lệ tiếp thị ngữ cảnh theo thời gian thực. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Cung cấp công cụ số trên LPBank Plus và LPBank Biz cho phép người dùng tùy chỉnh chọn số tài khoản iName, bật/tắt hạn mức giao dịch, chủ động đăng ký tài khoản Sinh lời Lộc Phát. Chưa công bố tỷ lệ khách hàng thực tế sử dụng các công cụ tùy chỉnh này. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6; https://vnba.org.vn/vi/emagazine/lpbank--hanh-trinh-vuon-minh-tro-thanh-ngan-hang-loc-phat-cua-moi-nha-17146.htm</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Minh chứng bằng số liệu hành vi thực tế của khách hàng: Năm 2024 thu hút hơn 1 triệu khách hàng mới đăng ký App LPBank; thực hiện 93,4 triệu giao dịch số với tổng giá trị trên 998.000 tỷ đồng; mảng thẻ đạt giải thưởng tăng trưởng doanh số Outstanding Payment Volume YoY Growth 2024 từ VISA. https://daidoanket.vn/dau-an-esg-cua-lpbank-tu-lanh-dao-xanh-chau-a-den-top-10-ngan-hang-viet-nam-xanh-10309415.html</x:t>
   </x:si>
   <x:si>
@@ -3388,15 +3382,6 @@
     <x:t xml:space="preserve">LPBank quán triệt giá trị cốt lõi "Khách hàng là trọng tâm" và xác định tầm nhìn chiến lược giai đoạn 2024–2028: "Trở thành TOP 1 Ngân hàng bán lẻ tại khu vực nông thôn và đô thị loại 2 trên nền tảng số, và TOP 5 dịch vụ Ngân hàng ưu tiên tại các đô thị lớn".https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Triển khai Dự án UI/UX cải tiến toàn diện giao diện LPBank Plus và LPBank Biz dựa trên nghiên cứu hành vi người dùng; thực hiện cải tổ bộ máy tinh gọn (giảm từ 17 Khối xuống 8 Khối) để chuyển dịch mô hình vận hành theo định hướng lấy khách hàng làm trọng tâm, làm nền tảng thay đổi tư duy thiết kế sản phẩm và phục vụ. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Dành nguồn vốn đầu tư lớn thực hiện hàng loạt dự án công nghệ hạ tầng cốt lõi: chuyển đổi Core Banking T24 (Temenos), vận hành hệ thống Kondor Treasury, phát triển Nền tảng số LPBank Biz, siêu ứng dụng LPBank Plus, Datalake, nâng cấp 02 Trung tâm dữ liệu (Data Center) mới và Tổng đài đa kênh thông minh IVR.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Triển khai 86 tính năng/sản phẩm mới trong năm 2024. Danh mục phủ rộng từ cá nhân (LPBank Plus, iName, tài khoản Lộc Phát, thẻ JCB Ultimate, mở tài khoản VNeID) đến doanh nghiệp (LPBank Biz hỗ trợ chuyển tiền lô 40.000 lệnh, phân quyền 5 cấp duyệt) và dịch vụ công/an sinh xã hội.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Mở tài khoản và định danh 100% online qua eKYC/VNeID của Bộ Công an; ứng dụng sinh trắc học theo Quyết định 2345/QĐ-NHNN; số hóa quy trình tín dụng BPM, tra cứu CIC tự động qua API (CIS), ứng dụng chữ ký số và tinh gọn danh mục hồ sơ tín dụng (thay thế sổ hộ khẩu giấy bằng kết nối VNeID/Cổng Dịch vụ công quốc gia).https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
@@ -3415,18 +3400,12 @@
     <x:t xml:space="preserve">Đưa vào vận hành hệ thống Core Banking T24 (Temenos), Datalake, Datawarehouse và kết nối làm sạch dữ liệu với Cơ sở dữ liệu quốc gia về dân cư (VNeID/C06 - Bộ Công an) tạo nguồn dữ liệu tin cậy duy nhất cho thông tin định danh (eKYC) và lịch sử giao dịch cốt lõi. BCTN chưa chứng minh được việc hợp nhất nguồn dữ liệu duy nhất trên toàn bộ các kênh phân phối và đối tác bên ngoài. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Phân tích nhu cầu theo từng nhóm khách hàng mục tiêu để thiết kế gói giải pháp riêng (Lộc Phát Pay cho hộ kinh doanh, Sinh lời Lộc Phát, gói tín dụng Hưu trí, cho vay phụ nữ hợp tác ADB). Đã bắt đầu ứng dụng AI/Big Data trên ứng dụng LPBank Plus để phân tích xu hướng tiêu dùng, nhưng chưa triển khai mô hình dự báo nhu cầu thời gian thực trên toàn hệ thống (Mức 4/5).https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Đổi tên thương mại thành Ngân hàng TMCP Lộc Phát Việt Nam gắn liền với giá trị cốt lõi "Chính trực". Thương hiệu được khẳng định qua xếp hạng tín nhiệm A+ (triển vọng Ổn định) từ VIS Rating (Moody's), Top 14 Ngân hàng có tầm quan trọng hệ thống (NHNN phê duyệt) và Top 50 Doanh nghiệp xuất sắc Việt Nam. Quy mô tiền gửi huy động đạt 338.662 tỷ đồng.https://lpbank.com.vn/api/content-file/public/file/view/cfbdb8c8-ff1c-4bd7-9dbe-00f3d41320a6</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Áp dụng và duy trì các chuẩn an toàn thông tin &amp; bảo mật quốc tế ISO/IEC 27001, PCI-DSS (bảo mật thẻ), SWIFT CSP; tuân thủ Nghị định 13/2023/NĐ-CP về bảo vệ dữ liệu cá nhân; tổ chức tập huấn an toàn thông tin &amp; bảo mật dữ liệu bắt buộc cho 100% cán bộ nhân viên. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Triển khai xác thực sinh trắc học bắt buộc theo Quyết định 2345/QĐ-NHNN từ 01/07/2024; tích hợp giải pháp liên kết định danh VNeID/C06 giúp ngăn chặn tài khoản giả mạo/lừa đảo; trang bị công nghệ bảo vệ ứng dụng (App Shielding) và phần mềm dò quét mã độc 24/7 trên LPBank Plus, LPBank Biz, E-Banking.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Chính thức đổi tên thương mại thành "Ngân hàng TMCP Lộc Phát Việt Nam" (NHNN phê duyệt QĐ 423/QĐ-TTGSNH2), ra mắt bộ nhận diện thương hiệu mới năng động và phát triển thương hiệu sub-brand riêng cho phân khúc LPBank Priority gắn với chiến lược bán lẻ 2024–2028. https://thanhtra.com.vn/thong-tin-doanh-nghiep-49F64E63D/dai-hoi-dong-co-dong-lpbank-doi-ten-ngan-hang-de-phu-hop-hon-voi-giai-doan-phat-trien-moi-4937E13E.html</x:t>
   </x:si>
   <x:si>
@@ -3439,33 +3418,18 @@
     <x:t xml:space="preserve">Tích hợp hệ sinh thái 512 phòng giao dịch bưu điện (Vietnam Post); ký kết hợp tác chính thức với Trung tâm RAR - Cục C06 (Bộ Công an) triển khai mở tài khoản trực tuyến và xác thực qua ứng dụng VNeID; kết nối hệ sinh thái Viettel Money và tài trợ chuỗi KHDN. https://lpbank.com.vn/tin-tuc/lpbank-trien-khai-dich-vu-mo-tai-khoan-thanh-toan-truc-tuyen-tren-vneid-cua-bo-cong-an/; https://kisvn.vn/san-pham-dich-vu/dich-vu-chung-khoan/trai-phieu-ngan-hang-lpb-3998</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Thiết kế hạ tầng API kết nối ứng dụng LPBank Plus và LPBank Biz với các cổng thanh toán (Napas, VISA, JCB), ví điện tử/thẻ ảo (Apple Pay, Google Wallet via Visa Tokenization) và hệ thống định danh VNeID. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Hợp tác với Temenos (Core T24 - trao giải "Triển khai Core Banking nhanh nhất Châu Á"); Ngân hàng Phát triển Châu Á ADB (giải ngân 3.301 tỷ đồng tài trợ nữ chủ doanh nghiệp); Vietnam Post; VISA (giải thưởng Outstanding Payment Volume YoY Growth 2024). https://vneconomy.vn/lpbank-huy-dong-thanh-cong-80-trieu-usd-tu-adb.htm; https://lpbank.com.vn/tin-tuc/lpbank-trien-khai-dich-vu-mo-tai-khoan-thanh-toan-truc-tuyen-tren-vneid-cua-bo-cong-an/</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Nhờ tự động hóa quy trình và chuyển đổi số, chỉ số chi phí trên thu nhập (CIR) giảm mạnh từ 36,86% xuống 29,15% (và giảm tiếp xuống 28,31% năm 2025); lợi nhuận trước thuế tăng 73% đạt 12.168 tỷ đồng; chỉ số sinh lời ROE đạt 25,10% thuộc Top đầu ngành. https://www.tinnhanhchungkhoan.vn/lpbank-lpb-cong-bo-bao-cao-tai-chinh-kiem-toan-nam-2024-loi-nhuan-tang-73-post366318.html; https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Liên tục nâng cấp và cho ra mắt các nền tảng số mới: bổ sung 86 tính năng mới năm 2024, ra mắt ứng dụng LPBank Biz cho KHDN (tháng 10/2024) và ứng dụng LPBank Plus tích hợp trợ lý AI chuyển tiền hội thoại LP Pay (tháng 3/2026). https://lpbank.com.vn/tin-tuc/lpbank-trien-khai-dich-vu-mo-tai-khoan-thanh-toan-truc-tuyen-tren-vneid-cua-bo-cong-an/</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Chủ động tinh gọn bộ máy theo chủ trương Chính phủ (giảm từ 17 Khối xuống 8 Khối); đáp ứng quy định sinh trắc học Quyết định 2345/QĐ-NHNN; đẩy mạnh tín dụng xanh (dư nợ 9.512 tỷ đồng); hoàn thành chuẩn mực rủi ro Basel III và IFRS 9. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Phân tích nhu cầu theo từng nhóm khách hàng mục tiêu (hộ kinh doanh Lộc Phát Pay, cán bộ hưu trí, lực lượng vũ trang, KHDN FDI) để thiết kế các gói giải pháp tài chính "may đo". Chưa công bố các báo cáo nghiên cứu khảo sát thị trường độc lập quy mô lớn. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Cân đối danh mục giữa sản phẩm thế mạnh truyền thống (cho vay nông nghiệp nông thôn 80.000 tỷ, tín dụng hưu trí) và các giải pháp số hóa (LPBank Plus, LPBank Biz, tài khoản Sinh lời Lộc Phát, iName, phái sinh/Kondor Treasury). https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Xác định lộ trình phát triển danh mục: bổ sung 86 tính năng năm 2024, ra mắt LPBank Biz (T10/2024), ra mắt LPBank Plus AI-first (T3/2026) và kế hoạch ra mắt thương hiệu sub-brand riêng cho LPBank Priority. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Đạt giải thưởng "Ngân hàng có sản phẩm dịch vụ sáng tạo tiêu biểu 2026" tại Giải thưởng Ngân hàng Việt Nam tiêu biểu; ra mắt thẻ quốc tế JCB Ultimate, gói Sinh lời tự động Lộc Phát, dịch vụ mở tài khoản VNeID và trợ lý AI chuyển tiền LP Pay. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Chiến lược giai đoạn 2024–2028 nhất quán với tầm nhìn: "TOP 1 Ngân hàng bán lẻ tại khu vực nông thôn và đô thị loại 2 trên nền tảng công nghệ số" và "TOP 5 dịch vụ ngân hàng ưu tiên tại các đô thị lớn". https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
@@ -3499,18 +3463,12 @@
     <x:t xml:space="preserve">Áp dụng giải pháp tiết kiệm điện năng trong vận hành máy chủ và tối ưu hiệu suất tiêu thụ năng lượng tại 02 Trung tâm dữ liệu (Data Center) mới. Tuy nhiên, BCTN chưa công bố chỉ số định lượng % điện năng tiết kiệm riêng của hệ thống CNTT. https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Chủ động tìm kiếm và áp dụng các công nghệ mới dẫn dắt thị trường: Trợ lý AI chuyển tiền bằng hội thoại (LP Pay), mô hình ngôn ngữ lớn LLM (Smart Nav) trên LPBank Plus, định danh sinh trắc học eKYC/NFC chip CCCD, Core T24 và Kondor Treasury.https://static2.vietstock.vn/vietstock/2025/4/9/20250409_lpb_250409_5__eng___report_of_ceo.pdf; https://lpbank.com.vn/tin-tuc/17-4-2024-thong-bao-chuyen-doi-he-thong-ngan-hang-loi-corebanking/; https://lpbank.com.vn/tin-tuc/lpbank-trien-khai-he-thong-kondor-treasury-nhanh-nhat-chau-a-thai-binh-duong/</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Quy hoạch lộ trình công nghệ gắn liền với mục tiêu chiến lược 2025–2028 ("Top 1 Ngân hàng bán lẻ số tại nông thôn &amp; đô thị loại 2; Top 5 Priority"), cụ thể hóa qua 04 Danh mục dự án CĐS trọng điểm.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Triển khai Core T24, Nền tảng LPBank Biz và tích hợp hệ thống theo kiến trúc hướng dịch vụ (SOA) kết nối giữa T24, Uniform, Antifraud, EWS, BPM. BCTN chưa chứng minh việc áp dụng 100% microservices/event-driven cho toàn bộ hệ thống ứng dụng cũ.https://lpbank.com.vn/tin-tuc/17-4-2024-thong-bao-chuyen-doi-he-thong-ngan-hang-loi-corebanking/; https://lpbank.com.vn/tin-tuc/chinh-thuc-ra-mat-nen-tang-so-lpbank-biz-danh-cho-doanh-nghiep/</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Cho phép cấu hình phân quyền linh hoạt 5 cấp duyệt, hạn mức chuyển tiền lô 40.000 lệnh trên LPBank Biz; tự tùy chỉnh tài khoản iName, chọn số tài khoản phong thủy trên LPBank Plus.https://lpbank.com.vn/doanh-nghiep/ngan-hang-so-doanh-nghiep</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Thiết kế hạ tầng Core T24, Kondor Treasury và hệ thống Datalake/Datawarehouse theo chuẩn Cloud-ready, sẵn sàng tích hợp và mở rộng trên hạ tầng đám mây.https://lpbank.com.vn/tin-tuc/lpbank-trien-khai-he-thong-kondor-treasury-nhanh-nhat-chau-a-thai-binh-duong/</x:t>
   </x:si>
   <x:si>
@@ -3523,18 +3481,12 @@
     <x:t xml:space="preserve">Tuân thủ quy định phân loại và bảo vệ hệ thống thông tin theo cấp độ của NHNN (Thông tư 09/2020/TT-NHNN); đầu tư trang bị hệ thống bảo mật toàn diện máy chủ tại 02 Trung tâm dữ liệu (Data Center) mới trang bị giải pháp DRP dự phòng thảm họa.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Cài đặt phần mềm dò quét mã độc 24/7 trên Ebanking, LPBank Biz, LPBank Plus, Core T24; triển khai dự án Pentest (đánh giá xâm nhập kiểm thử), nâng cấp hệ thống Internet tập trung Forcepoint V5000 và giám sát an ninh mạng 24/7.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Thành lập Tổ công tác đặc biệt ứng phó sự cố an ninh mạng; phối hợp với NHNN và VNISA; duy trì chứng chỉ bảo mật quốc tế SWIFT CSP giảm thiểu gian lận giao dịch quốc tế và đào tạo an toàn thông tin bắt buộc cho 100% cán bộ nhân viên.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Hoàn thiện Hệ thống lưu trữ camera an ninh và Hệ thống phòng chống tấn công ATM/CDM tại 100% điểm ATM; kiểm soát an ninh vật lý nghiêm ngặt tại Trụ sở chính LPB Tower và 2 Data Center.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Tích hợp Generative AI/Agentic AI (trợ lý LP Pay) và LLM (Smart Nav) trên ứng dụng LPBank Plus; ứng dụng công nghệ IVR nhận diện giọng nói tại Tổng đài CSKH và AI phân tích dữ liệu cảnh báo rủi ro sớm (EWS).https://static2.vietstock.vn/vietstock/2025/4/9/20250409_lpb_250409_5__eng___report_of_ceo.pdf</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Thiết lập và vận hành hệ thống Datalake và Datawarehouse tập trung; ứng dụng phân tích Dữ liệu lớn (Big Data) để phát hiện biến động tín dụng, nợ xấu và xu hướng thị trường.https://lpbank.com.vn/tin-tuc/lpbank-trien-khai-he-thong-kondor-treasury-nhanh-nhat-chau-a-thai-binh-duong/</x:t>
   </x:si>
   <x:si>
@@ -3559,9 +3511,6 @@
     <x:t xml:space="preserve">Triển khai phần mềm "Quản lý tài sản tập trung toàn hàng" cho phép theo dõi lịch sử biến động, kiểm kê và truy vết vòng đời thiết bị CNTT; vận hành ổn định 02 Data Center đáp ứng 93,4 triệu giao dịch số.https://daidoanket.vn/dau-an-esg-cua-lpbank-tu-lanh-dao-xanh-chau-a-den-top-10-ngan-hang-viet-nam-xanh-10309415.html</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Sử dụng hạ tầng đám mây (Cloud-ready/Private Cloud) phục vụ lưu trữ tài liệu, vận hành Datalake và ứng dụng ngân hàng số LPBank Plus/LPBiz.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Tự động hóa quy trình phê duyệt tín dụng BPM, tự động phân luồng giọng nói IVR, tự động báo nguồn &amp; kiểm tra hạn mức thanh toán quốc tế, tự động hóa báo cáo Dashboard 4 chiều.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
@@ -3574,24 +3523,15 @@
     <x:t xml:space="preserve">Triển khai phần mềm "Quản lý tài sản tập trung toàn hàng" cho phép theo dõi chi tiết lịch sử biến động, kiểm kê, truy vết lịch sử vòng đời tài sản; kết hợp bảo hiểm gian lận và kế hoạch duy trì kinh doanh liên tục BCP.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Thực hiện Dự án UI/UX cải tiến toàn diện giao diện sản phẩm trên LPBank Plus và LPBank Biz dựa trên nghiên cứu mô hình "3S" (Simple-Smart-Safe), đổi mới giao diện Website chuẩn hóa nhận diện thương hiệu.https://lpbank.com.vn/tin-tuc/17-6-2024-nen-tang-ngan-hang-so-lienviet24h-doi-ten-thanh-lpbank/</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Áp dụng phương pháp triển khai dự án thần tốc và linh hoạt, hoàn thành đưa vào vận hành Core T24 trong 7 tháng (Temenos vinh danh "Triển khai Core Banking nhanh nhất Châu Á") và hệ thống Kondor Treasury trong 6 tháng (nhanh nhất khu vực Châu Á - Thái Bình Dương). https://www.finastra.com/press-media/finastra-and-lpbank-modernize-treasury-management-operations-record-time; https://static2.vietstock.vn/vietstock/2025/4/9/20250409_lpb_250409_5__eng___report_of_ceo.pdf</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Được trao giải thưởng "Ngân hàng có sản phẩm dịch vụ sáng tạo tiêu biểu 2026" tại Giải thưởng Ngân hàng Việt Nam tiêu biểu; ra mắt thẻ Visa Tokenization, trợ lý AI chuyển tiền LP Pay, mở tài khoản VNeID và gói Combo Lộc Phát.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Hợp tác chiến lược với Temenos (Core T24), Trung tâm RAR - C06 Bộ Công an (mở tài khoản VNeID), Vietnam Post (bưu điện số &amp; an sinh xã hội), Ngân hàng Phát triển Châu Á ADB (tín dụng phụ nữ), VISA, JCB, Viettel Digital.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Quản lý thành công đợt tái cấu trúc tinh gọn mô hình từ 17 Khối xuống 8 Khối; tổ chức 261 chương trình/khóa đào tạo với 324.933 lượt học viên, số hóa 100% tài liệu quy trình mới trên e-learning giúp hệ thống vận hành thông suốt.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Kiểm soát quy trình phát hành golive an toàn cho các hệ thống lớn: Kondor Treasury (golive T4/2024), Core T24 (golive T5/2024), LPBank Biz (T10/2024), LPBank Plus (T3/2026) đảm bảo không gây gián đoạn dịch vụ 24/7.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Duy trì vận hành ổn định 24/7 hệ thống giao dịch số xử lý 93,4 triệu giao dịch với tổng giá trị trên 998.000 tỷ đồng; cắt giảm chỉ số CIR xuống 29,15% khẳng định hiệu quả vận hành tối ưu.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
   </x:si>
   <x:si>
@@ -3604,12 +3544,6 @@
     <x:t xml:space="preserve">Vận hành Hệ thống Phân tích lợi nhuận đa chiều toàn diện (MPA) đo lường và đánh giá lợi nhuận chi tiết đến từng khách hàng, sản phẩm, cán bộ bán hàng, kênh phân phối và vùng địa lý. https://nhadautu.vn/lpbank-va-ey-consulting-vn-ky-hop-dong-tu-van-va-trien-khai-he-thong-do-luong-loi-nhuan-da-chieu-d83663.html</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Triển khai xác thực sinh trắc học Quyết định 2345/QĐ-NHNN; vận hành phần mềm phòng chống gian lận Antifraud, phần mềm Fico Tonbeller, cài đặt phần mềm dò quét mã độc 24/7 và công nghệ App Shielding trên LPBank Plus.https://lpbank.com.vn/tin-tuc/lpbank-trien-khai-xac-thuc-giao-dich-bang-sinh-trac-hoc-tren-ung-dung-ngan-hang-so/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Vận hành ổn định hệ thống Core T24, Kondor Treasury, ứng dụng LPBiz/LPBank Plus và 02 Trung tâm dữ liệu (Data Center) mới trang bị giải pháp giám sát 24/7 và phòng thủ an ninh mạng Forcepoint V5000.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Tỷ lệ CBNV nữ đạt 59,72%, tỷ lệ cán bộ quản lý nữ đạt 32,83%; trang bị phòng y tế và phòng chức năng riêng cho nhân viên nữ nuôi con nhỏ; thực hiện chính sách đãi ngộ không phân biệt giới tính.https://cafef1.mediacdn.vn/download/210425/lpb-bao-cao-thuong-nien-nam-2024-0.pdf</x:t>
   </x:si>
   <x:si>
@@ -3643,9 +3577,6 @@
     <x:t xml:space="preserve">LPBank triển khai xây dựng và duy trì từ điển dữ liệu chuẩn hóa (Data Dictionary), hệ thống phân loại và tổ chức dữ liệu trong khuôn khổ Quản trị dữ liệu ESG và các dự án làm giàu dữ liệu tập trung Datalake/Datawarehouse.https://lpbank.com.vn/tin-tuc/3235-lpbank-plus-ung-dung-ngan-hang-so-the-he-moi-tich-hop-tro-ly-ai-chuyen-tien-bang-hoi-thoai; https://en.vneconomy.vn/bao-cao-phat-trien-ben-vung-cua-lpbank-co-gi.htm</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Duy trì các chứng chỉ an toàn thông tin &amp; bảo mật quốc tế ISO/IEC 27001, PCI-DSS (bảo mật thẻ), SWIFT CSP; trang bị phần mềm dò quét mã độc 24/7 trên Ebanking, LPBank Biz, LPBank Plus, Core T24, AD, LIM và ứng dụng công nghệ App Shielding.https://lpbank.com.vn/api/content-file/public/file/view/5bb2a4bb-a070-415a-8eea-54b36c848de6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Ban hành Khung quản trị dữ liệu thiết lập các nguyên tắc và cơ chế thống nhất triển khai quản trị dữ liệu từ Hội sở đến đơn vị kinh doanh; ban hành quy định an toàn thông tin &amp; bảo mật dữ liệu.https://en.vneconomy.vn/bao-cao-phat-trien-ben-vung-cua-lpbank-co-gi.htm; https://www.scribd.com/document/725622501/LPB</x:t>
   </x:si>
   <x:si>
@@ -3665,9 +3596,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Ban Điều hành sử dụng hệ thống báo cáo Dashboard 4 chiều, Hệ thống Phân tích lợi nhuận đa chiều (MPA) và công cụ cảnh báo rủi ro sớm (EWS, ALM) để ra quyết định kinh doanh và điều chỉnh chính sách tín dụng/lãi suất kịp thời.https://nhadautu.vn/lpbank-va-ey-consulting-vn-ky-hop-dong-tu-van-va-trien-khai-he-thong-do-luong-loi-nhuan-da-chieu-d83663.html</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ứng dụng AI và Big Data phân tích khối lượng lớn dữ liệu giao dịch phát hiện rủi ro sớm (EWS); vận hành ứng dụng LPBank Plus phát triển theo định hướng AI-first tích hợp trợ lý hội thoại LP Pay và Smart Nav; tích hợp phần mềm Antifraud.https://lpbank.com.vn/tin-tuc/3235-lpbank-plus-ung-dung-ngan-hang-so-the-he-moi-tich-hop-tro-ly-ai-chuyen-tien-bang-hoi-thoai; https://tudonghoangaynay.vn/lpbank-tien-phong-chuyen-doi-so-kien-tao-he-sinh-thai-tai-chinh-hien-dai-14065.html</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Chưa thấy báo cáo đo lường trực tiếp mức độ 'hứng thú' của khách hàng theo định nghĩa tiêu chí DBI; CSAT đo sự hài lòng, không đồng nhất với hứng thú.</x:t>
@@ -4154,9 +4082,6 @@
     <x:t xml:space="preserve">Ngân hàng tích hợp VNeID để chi trả an sinh, hợp tác với các địa phương về thanh toán dịch vụ công và phương tiện giao thông, mở rộng liên kết ngoài ngân hàng.https://saigonbank.com.vn/vi/tin-tuc/Tin-tuc-ngan-hang/VNIED2; https://www.saigonbank.com.vn/vi/tin-tuc/Tin-tuc-ngan-hang/Kiosk</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Kế hoạch 2026 xác định phát triển hệ sinh thái thanh toán qua tài khoản SAIGONBANK và kết nối dịch vụ y tế, giáo dục, hành chính công; mới là định hướng công bố.https://saigonbank.com.vn/vi/tin-tuc/Tin-tuc-ngan-hang/SGBHDHDCD26</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Chưa tìm thấy thông tin công khai đủ cụ thể để xác minh tiêu chí «Lựa chọn đối tác» theo thang DBI. Mức 0 thể hiện thiếu bằng chứng để chấm, KHÔNG kết luận SAIGONBANK không thực hiện.</x:t>
   </x:si>
   <x:si>
@@ -4181,15 +4106,9 @@
     <x:t xml:space="preserve">Chưa tìm thấy thông tin công khai đủ cụ thể để xác minh tiêu chí «Cân đối danh mục sản phẩm và dịch vụ» theo thang DBI. Mức 0 thể hiện thiếu bằng chứng để chấm, KHÔNG kết luận SAIGONBANK không thực hiện.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">SAIGONBANK nêu kế hoạch bổ sung tiện ích ngân hàng số, thanh toán hiện đại và số hóa quy trình cấp tín dụng trong giải pháp phát triển năm 2026.https://saigonbank.com.vn/vi/tin-tuc/Tin-tuc-ngan-hang/SGBHDHDCD26; https://vnba.org.vn/vi/saigonbank-dat-muc-tieu-loi-nhuan-truoc-thue-310-ty-dong-trong-2026-21403.htm</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Từ 2023 đến 2025, ngân hàng mở eKYC, thêm tiện ích Smart Banking/PAY, thanh toán không tiếp xúc và kết nối VNeID.https://www.saigonbank.com.vn/vi/tin-tuc/Tin-tuc-ngan-hang/Mo-tai-khoan-truc-tuyen-chi-vai-phut-tren-ung-dung-SAIGONBANK-Smart-Banking-1</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">BCTN 2025–2026 đặt chuyển đổi số theo lộ trình phù hợp làm nền tảng phát triển sản phẩm dịch vụ; chiến lược đang được cụ thể hóa.https://static2.vietstock.vn/data/HNX/2025/BCTN/VN/SGB_Baocaothuongnien_2025/1_sgb_2026_4_20_43bf2b9_vi_baocaothuongnien_2025_compressedda_ky.pdf</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Quyết định 479 thành lập Trung tâm Chuyển đổi số trực thuộc ngân hàng, giao nhiệm vụ tham mưu, phát triển và vận hành sản phẩm số phối hợp với định hướng kinh doanh.https://www.saigonbank.com.vn/vi/tin-tuc/Tin-tuc-ngan-hang/SGBCDS; https://www.saigonbank.com.vn/vi/quan-he-co-dong/Cong-bo-thong-tin/chuyendoitrungtamkinhdoanhthe</x:t>
   </x:si>
   <x:si>
@@ -4199,9 +4118,6 @@
     <x:t xml:space="preserve">SAIGONBANK vận hành kiểm soát rủi ro theo Basel II, triển khai hệ thống xếp hạng tín dụng nội bộ/cảnh báo sớm và ban hành 18 chính sách quản lý rủi ro trong 2025.https://www.saigonbank.com.vn/files/File/Quan-He-Co-Dong/Bao-Cao-Thuong-Nien/T0426/Bao-cao-thuong-nien-SAIGONBANK-nam-2025.pdf</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Định hướng 2026 nêu triển khai chuyển đổi số theo lộ trình; Quyết định 479 xác lập đầu mối tổ chức, nhưng chưa công bố lộ trình chi tiết theo giai đoạn/toàn đơn vị.https://saigonbank.com.vn/vi/tin-tuc/Tin-tuc-ngan-hang/SGBHDHDCD26</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Thành lập Trung tâm Chuyển đổi số, bổ sung dịch vụ PAY/Smart Banking, VNeID và thanh toán số cho thấy chiến lược đã được triển khai ở các mảng trọng tâm.https://www.saigonbank.com.vn/vi/tin-tuc/Tin-tuc-ngan-hang/SGBCDS</x:t>
   </x:si>
   <x:si>
@@ -4224,9 +4140,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Ứng dụng eKYC, sinh trắc học, VNeID, Kiosk thông minh; nâng cấp Oracle 19C, giám sát truy cập NAC và tường lửa WAF.https://saigonbank.com.vn/vi/tin-tuc/Tin-tuc-ngan-hang/VNIED2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Kế hoạch 2026 gắn đầu tư công nghệ, bảo mật và hạ tầng số với mục tiêu nâng cao chất lượng dịch vụ, phù hợp một phần chiến lược kinh doanh.https://saigonbank.com.vn/vi/tin-tuc/Tin-tuc-ngan-hang/SGBHDHDCD26</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Chưa tìm thấy thông tin công khai đủ cụ thể để xác minh tiêu chí «Kiến trúc Microservices &amp; kiến trúc theo hướng dịch vụ (SOA - Service-Oriented Architecture)» theo thang DBI. Mức 0 thể hiện thiếu bằng chứng để chấm, KHÔNG kết luận SAIGONBANK không thực hiện.</x:t>
@@ -4570,10 +4483,13 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="2">
+  <x:cellXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -14887,7 +14803,7 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="2" hidden="1">
+    <row r="2" ht="336" hidden="1" customHeight="1">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -14903,8 +14819,14 @@
       <c r="E2">
         <v>2</v>
       </c>
-      <c r="F2" t="s">
-        <v>1115</v>
+      <c r="F2" s="2" t="str">
+        <v>Năm 2024, LPBank triển khai giao diện ứng dụng mới, dịch vụ iName và tài khoản số đẹp. BCTN 2025 mô tả thiết kế sản phẩm, chính sách và trải nghiệm dựa trên hành trình, phân khúc khách hàng. Các nội dung này thể hiện những khía cạnh cá nhân hóa trong kỳ 2023–2025.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 25 (trang in 48–49)
+Trích đoạn: “Hơn 1 triệu Khách hàng đăng ký mới app LPBank, 86 tính năng sản phẩm mới được triển khai”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=25
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 26 (trang in 50–51)
+Trích đoạn: “Sản phẩm, chính sách, mô hình phục vụ, mô hình vận hành và trải nghiệm được thiết kế dựa trên hành trình khách hàng”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=26</v>
       </c>
     </row>
     <row r="3" hidden="1">
@@ -14924,10 +14846,10 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>1116</v>
-      </c>
-    </row>
-    <row r="4" hidden="1">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="4" ht="196" hidden="1" customHeight="1">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -14943,8 +14865,11 @@
       <c r="E4">
         <v>2</v>
       </c>
-      <c r="F4" t="s">
-        <v>1117</v>
+      <c r="F4" s="2" t="str">
+        <v>BCTN 2024 ghi nhận dịch vụ iName và tài khoản số đẹp trên kênh số, cùng giao diện ứng dụng được cải tiến. Đây là những lựa chọn giúp khách hàng tùy chỉnh tên hoặc số tài khoản trong giai đoạn nghiên cứu.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 25 (trang in 48–49)
+Trích đoạn: “Hơn 1 triệu Khách hàng đăng ký mới app LPBank, 86 tính năng sản phẩm mới được triển khai”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=25</v>
       </c>
     </row>
     <row r="5" hidden="1">
@@ -14984,7 +14909,7 @@
         <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="7" hidden="1">
@@ -15004,7 +14929,7 @@
         <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="8" hidden="1">
@@ -15024,7 +14949,7 @@
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="9" hidden="1">
@@ -15044,7 +14969,7 @@
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="10" hidden="1">
@@ -15064,7 +14989,7 @@
         <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="11" hidden="1">
@@ -15084,10 +15009,10 @@
         <v>4</v>
       </c>
       <c r="F11" t="s">
-        <v>1123</v>
-      </c>
-    </row>
-    <row r="12" hidden="1">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="12" ht="336" hidden="1" customHeight="1">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -15103,11 +15028,17 @@
       <c r="E12">
         <v>4</v>
       </c>
-      <c r="F12" t="s">
-        <v>1124</v>
-      </c>
-    </row>
-    <row r="13" hidden="1">
+      <c r="F12" s="2" t="str">
+        <v>Năm 2024, LPBank thực hiện dự án UI/UX để tối ưu giao diện ứng dụng ngân hàng số. BCTN 2025 nêu sản phẩm, chính sách, mô hình phục vụ, mô hình vận hành và trải nghiệm được thiết kế dựa trên hành trình khách hàng trên cả kênh số và kênh vật lý.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 34 (trang in 66–67)
+Trích đoạn: “Dự án UI/UX: Tối ưu giao diện sản phẩm nhằm nâng cao trải nghiệm Khách hàng trên kênh ứng dụng ngân hàng số LPBank.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=34
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 26 (trang in 50–51)
+Trích đoạn: “Sản phẩm, chính sách, mô hình phục vụ, mô hình vận hành và trải nghiệm được thiết kế dựa trên hành trình khách hàng”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=26</v>
+      </c>
+    </row>
+    <row r="13" ht="336" hidden="1" customHeight="1">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -15123,11 +15054,17 @@
       <c r="E13">
         <v>4</v>
       </c>
-      <c r="F13" t="s">
-        <v>1125</v>
-      </c>
-    </row>
-    <row r="14" hidden="1">
+      <c r="F13" s="2" t="str">
+        <v>BCTN 2024 ghi nhận đầu tư nguồn lực cho bốn danh mục dự án: phát triển khách hàng, vận hành tinh gọn, nâng cao trải nghiệm khách hàng và số hóa quản lý rủi ro. Các dự án gồm CoreBanking T24, Kondor Treasury, LPBank Biz, UI/UX và tổng đài đa kênh.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 33 (trang in 64–65)
+Trích đoạn: “Trong năm 2024, LPBank đã triển khai nhiều dự án trọng điểm tập trung vào 04 Danh mục dự án”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=33
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 32 (trang in 62–63)
+Trích đoạn: “Sau thời gian triển khai chỉ 7 tháng, LPBank đã đưa vào hoạt động ổn định giải pháp ngân hàng lõi CoreBanking T24.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=32</v>
+      </c>
+    </row>
+    <row r="14" ht="409" hidden="1" customHeight="1">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -15143,8 +15080,17 @@
       <c r="E14">
         <v>4</v>
       </c>
-      <c r="F14" t="s">
-        <v>1126</v>
+      <c r="F14" s="2" t="str">
+        <v>Năm 2024, LPBank triển khai 86 tính năng/sản phẩm mới trên kênh số và ra mắt LPBank Biz ngày 03/10/2024. Năm 2025, ngân hàng phát triển giải pháp theo phân khúc và mô hình LPBank Priority, mở rộng danh mục phục vụ khách hàng cá nhân và doanh nghiệp.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 25 (trang in 48–49)
+Trích đoạn: “Hơn 1 triệu Khách hàng đăng ký mới app LPBank, 86 tính năng sản phẩm mới được triển khai”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=25
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 32 (trang in 62–63)
+Trích đoạn: “Sau thời gian triển khai chỉ 7 tháng, LPBank đã đưa vào hoạt động ổn định giải pháp ngân hàng lõi CoreBanking T24.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=32
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 27 (trang in 52–53)
+Trích đoạn: “Thiết kế giải pháp theo phân khúc. Ưu tiên giải pháp Combo để một điểm chạm khách hàng được dùng nhiều sản phẩm”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=27</v>
       </c>
     </row>
     <row r="15" hidden="1">
@@ -15164,7 +15110,7 @@
         <v>4</v>
       </c>
       <c r="F15" t="s">
-        <v>1127</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="16" hidden="1">
@@ -15184,7 +15130,7 @@
         <v>4</v>
       </c>
       <c r="F16" t="s">
-        <v>1128</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="17" hidden="1">
@@ -15204,7 +15150,7 @@
         <v>3</v>
       </c>
       <c r="F17" t="s">
-        <v>1129</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="18" hidden="1">
@@ -15224,7 +15170,7 @@
         <v>4</v>
       </c>
       <c r="F18" t="s">
-        <v>1130</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="19" hidden="1">
@@ -15244,7 +15190,7 @@
         <v>2</v>
       </c>
       <c r="F19" t="s">
-        <v>1131</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="20" hidden="1">
@@ -15264,10 +15210,10 @@
         <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>1132</v>
-      </c>
-    </row>
-    <row r="21" hidden="1">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="21" ht="350" hidden="1" customHeight="1">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -15283,8 +15229,14 @@
       <c r="E21">
         <v>2</v>
       </c>
-      <c r="F21" t="s">
-        <v>1133</v>
+      <c r="F21" s="2" t="str">
+        <v>BCTN 2025 mô tả giải pháp theo nhu cầu, hành vi khách hàng: giao dịch hằng ngày, tích lũy, vay vốn, bảo vệ và đầu tư. Cùng năm, LPBank công bố các dự án AI dự báo khách hàng ngừng sử dụng sản phẩm, cảnh báo sớm nợ xấu và học máy phân tích hành vi.
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 27 (trang in 52–53)
+Trích đoạn: “Thiết kế giải pháp theo phân khúc. Ưu tiên giải pháp Combo để một điểm chạm khách hàng được dùng nhiều sản phẩm”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=27
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 36 (trang in 70–71)
+Trích đoạn: “Nâng cấp nền tảng Mobile App thế hệ mới (Microservices + Hybrid Cloud): Tăng hiệu năng, khả năng mở rộng, góp phần nâng tỷ lệ giao dịch số lên 78%.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=36</v>
       </c>
     </row>
     <row r="22" hidden="1">
@@ -15304,7 +15256,7 @@
         <v>3</v>
       </c>
       <c r="F22" t="s">
-        <v>1134</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="23" hidden="1">
@@ -15344,10 +15296,10 @@
         <v>3</v>
       </c>
       <c r="F24" t="s">
-        <v>1135</v>
-      </c>
-    </row>
-    <row r="25" hidden="1">
+        <v>1129</v>
+      </c>
+    </row>
+    <row r="25" ht="350" hidden="1" customHeight="1">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -15363,8 +15315,14 @@
       <c r="E25">
         <v>4</v>
       </c>
-      <c r="F25" t="s">
-        <v>1136</v>
+      <c r="F25" s="2" t="str">
+        <v>Năm 2024, LPBank triển khai xác thực sinh trắc học theo Quyết định 2345 từ ngày 01/07/2024. Ngân hàng cài đặt phần mềm dò quét mã độc trên Ebanking, LPBank Biz, Core Banking, App LPBank, AD và hệ thống xác thực LIM để bảo vệ hệ thống, thông tin và giao dịch.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 34 (trang in 66–67)
+Trích đoạn: “Dự án UI/UX: Tối ưu giao diện sản phẩm nhằm nâng cao trải nghiệm Khách hàng trên kênh ứng dụng ngân hàng số LPBank.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=34
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Triển khai cài đặt phần mềm dò quét trên các hệ thống dịch vụ đặc biệt quan trọng, có nguy cơ gây thất thoát tiền hoặc thông tin”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=35</v>
       </c>
     </row>
     <row r="26" hidden="1">
@@ -15404,7 +15362,7 @@
         <v>3</v>
       </c>
       <c r="F27" t="s">
-        <v>1137</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="28" hidden="1">
@@ -15424,7 +15382,7 @@
         <v>3</v>
       </c>
       <c r="F28" t="s">
-        <v>1138</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="29" hidden="1">
@@ -15444,7 +15402,7 @@
         <v>4</v>
       </c>
       <c r="F29" t="s">
-        <v>1139</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="30" hidden="1">
@@ -15484,10 +15442,10 @@
         <v>3</v>
       </c>
       <c r="F31" t="s">
-        <v>1140</v>
-      </c>
-    </row>
-    <row r="32" hidden="1">
+        <v>1133</v>
+      </c>
+    </row>
+    <row r="32" ht="350" hidden="1" customHeight="1">
       <c r="A32" t="s">
         <v>189</v>
       </c>
@@ -15503,8 +15461,14 @@
       <c r="E32">
         <v>3</v>
       </c>
-      <c r="F32" t="s">
-        <v>1141</v>
+      <c r="F32" s="2" t="str">
+        <v>BCTN 2024 mô tả các dự án Visa Token tích hợp ví điện tử và các giải pháp kết nối hệ thống. BCTN 2025 ghi nhận triển khai Open API và Kong Enterprise để tích hợp đối tác, thúc đẩy Open Banking; báo cáo công bố thời gian tích hợp đối tác giảm 70%.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 33 (trang in 64–65)
+Trích đoạn: “Trong năm 2024, LPBank đã triển khai nhiều dự án trọng điểm tập trung vào 04 Danh mục dự án”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=33
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 36 (trang in 70–71)
+Trích đoạn: “Nâng cấp nền tảng Mobile App thế hệ mới (Microservices + Hybrid Cloud): Tăng hiệu năng, khả năng mở rộng, góp phần nâng tỷ lệ giao dịch số lên 78%.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=36</v>
       </c>
     </row>
     <row r="33" hidden="1">
@@ -15524,7 +15488,7 @@
         <v>4</v>
       </c>
       <c r="F33" t="s">
-        <v>1142</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="34" hidden="1">
@@ -15564,10 +15528,10 @@
         <v>4</v>
       </c>
       <c r="F35" t="s">
-        <v>1143</v>
-      </c>
-    </row>
-    <row r="36" hidden="1">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="36" ht="350" hidden="1" customHeight="1">
       <c r="A36" t="s">
         <v>189</v>
       </c>
@@ -15583,8 +15547,14 @@
       <c r="E36">
         <v>3</v>
       </c>
-      <c r="F36" t="s">
-        <v>1144</v>
+      <c r="F36" s="2" t="str">
+        <v>LPBank ghi nhận 86 tính năng/sản phẩm mới triển khai năm 2024. Năm 2025, Khối Công nghệ Thông tin vận hành mô hình quản trị dự án tập trung để điều phối toàn bộ dự án chuyển đổi số; tỷ lệ dự án hoàn thành go-live và đúng tiến độ được báo cáo là 88%.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 25 (trang in 48–49)
+Trích đoạn: “Hơn 1 triệu Khách hàng đăng ký mới app LPBank, 86 tính năng sản phẩm mới được triển khai”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=25
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Năm 2025, Khối Công nghệ Thông tin đã vận hành mô hình quản trị dự án tập trung để điều phối toàn bộ dự án chuyển đổi số.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=35</v>
       </c>
     </row>
     <row r="37" hidden="1">
@@ -15604,7 +15574,7 @@
         <v>3</v>
       </c>
       <c r="F37" t="s">
-        <v>1145</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="38" hidden="1">
@@ -15624,7 +15594,7 @@
         <v>2</v>
       </c>
       <c r="F38" t="s">
-        <v>1146</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="39" hidden="1">
@@ -15647,7 +15617,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="40" hidden="1">
+    <row r="40" ht="336" hidden="1" customHeight="1">
       <c r="A40" t="s">
         <v>189</v>
       </c>
@@ -15663,11 +15633,17 @@
       <c r="E40">
         <v>3</v>
       </c>
-      <c r="F40" t="s">
-        <v>1147</v>
-      </c>
-    </row>
-    <row r="41" hidden="1">
+      <c r="F40" s="2" t="str">
+        <v>BCTN 2025 mô tả chuyển từ cung cấp sản phẩm đơn lẻ sang combo giải pháp theo phân khúc, đồng thời tối ưu danh mục theo giá trị khách hàng và hiệu quả sử dụng vốn. Danh mục số trong kỳ có ứng dụng LPBank, LPBank Biz và các giải pháp phục vụ hoạt động nguồn vốn.
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 27 (trang in 52–53)
+Trích đoạn: “Thiết kế giải pháp theo phân khúc. Ưu tiên giải pháp Combo để một điểm chạm khách hàng được dùng nhiều sản phẩm”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=27
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 32 (trang in 62–63)
+Trích đoạn: “Sau thời gian triển khai chỉ 7 tháng, LPBank đã đưa vào hoạt động ổn định giải pháp ngân hàng lõi CoreBanking T24.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=32</v>
+      </c>
+    </row>
+    <row r="41" ht="336" hidden="1" customHeight="1">
       <c r="A41" t="s">
         <v>189</v>
       </c>
@@ -15683,11 +15659,17 @@
       <c r="E41">
         <v>3</v>
       </c>
-      <c r="F41" t="s">
-        <v>1148</v>
-      </c>
-    </row>
-    <row r="42" hidden="1">
+      <c r="F41" s="2" t="str">
+        <v>BCTN 2024 xác định bốn danh mục dự án chuyển đổi số gắn với khách hàng, vận hành, trải nghiệm và quản lý rủi ro. BCTN 2025 mô tả chuyển dịch danh mục bán lẻ sang giải pháp theo phân khúc, combo sản phẩm và quản trị vòng đời khách hàng.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 33 (trang in 64–65)
+Trích đoạn: “Trong năm 2024, LPBank đã triển khai nhiều dự án trọng điểm tập trung vào 04 Danh mục dự án”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=33
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 27 (trang in 52–53)
+Trích đoạn: “Thiết kế giải pháp theo phân khúc. Ưu tiên giải pháp Combo để một điểm chạm khách hàng được dùng nhiều sản phẩm”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=27</v>
+      </c>
+    </row>
+    <row r="42" ht="364" hidden="1" customHeight="1">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -15703,8 +15685,14 @@
       <c r="E42">
         <v>4</v>
       </c>
-      <c r="F42" t="s">
-        <v>1149</v>
+      <c r="F42" s="2" t="str">
+        <v>BCTN 2025 mô tả việc tái cấu trúc phương thức vận hành và tư duy tăng trưởng của Ngân hàng Bán lẻ: thiết kế giải pháp theo phân khúc, combo sản phẩm và quản trị danh mục/vòng đời khách hàng. Ngân hàng cũng công bố mô hình quản trị dự án tập trung cho toàn bộ dự án chuyển đổi số trong năm 2025.
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 27 (trang in 52–53)
+Trích đoạn: “Thiết kế giải pháp theo phân khúc. Ưu tiên giải pháp Combo để một điểm chạm khách hàng được dùng nhiều sản phẩm”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=27
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Năm 2025, Khối Công nghệ Thông tin đã vận hành mô hình quản trị dự án tập trung để điều phối toàn bộ dự án chuyển đổi số.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=35</v>
       </c>
     </row>
     <row r="43" hidden="1">
@@ -15724,7 +15712,7 @@
         <v>4</v>
       </c>
       <c r="F43" t="s">
-        <v>1150</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="44" hidden="1">
@@ -15744,7 +15732,7 @@
         <v>3</v>
       </c>
       <c r="F44" t="s">
-        <v>1151</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="45" hidden="1">
@@ -15764,7 +15752,7 @@
         <v>1</v>
       </c>
       <c r="F45" t="s">
-        <v>1152</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="46" hidden="1">
@@ -15784,7 +15772,7 @@
         <v>3</v>
       </c>
       <c r="F46" t="s">
-        <v>1153</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="47" hidden="1">
@@ -15804,7 +15792,7 @@
         <v>3</v>
       </c>
       <c r="F47" t="s">
-        <v>1154</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="48" hidden="1">
@@ -15824,7 +15812,7 @@
         <v>4</v>
       </c>
       <c r="F48" t="s">
-        <v>1155</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -15844,7 +15832,7 @@
         <v>4</v>
       </c>
       <c r="F49" t="s">
-        <v>1156</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -15884,7 +15872,7 @@
         <v>3</v>
       </c>
       <c r="F51" t="s">
-        <v>1157</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -15904,7 +15892,7 @@
         <v>4</v>
       </c>
       <c r="F52" t="s">
-        <v>1158</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="53" hidden="1">
@@ -15924,7 +15912,7 @@
         <v>3</v>
       </c>
       <c r="F53" t="s">
-        <v>1159</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="54" hidden="1">
@@ -15944,10 +15932,10 @@
         <v>2</v>
       </c>
       <c r="F54" t="s">
-        <v>1160</v>
-      </c>
-    </row>
-    <row r="55" hidden="1">
+        <v>1148</v>
+      </c>
+    </row>
+    <row r="55" ht="364" hidden="1" customHeight="1">
       <c r="A55" t="s">
         <v>364</v>
       </c>
@@ -15963,8 +15951,14 @@
       <c r="E55">
         <v>4</v>
       </c>
-      <c r="F55" t="s">
-        <v>1161</v>
+      <c r="F55" s="2" t="str">
+        <v>Trong năm 2024, LPBank đưa CoreBanking T24 và Kondor Treasury vào vận hành, đồng thời ra mắt LPBank Biz. BCTN 2025 ghi nhận các dự án Microservices, Hybrid Cloud, Open API/Kong Enterprise, Data Lakehouse, Customer 360/CDP và AI ứng dụng vào dự báo, quản lý rủi ro, chăm sóc khách hàng.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 32 (trang in 62–63)
+Trích đoạn: “Sau thời gian triển khai chỉ 7 tháng, LPBank đã đưa vào hoạt động ổn định giải pháp ngân hàng lõi CoreBanking T24.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=32
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 36 (trang in 70–71)
+Trích đoạn: “Nâng cấp nền tảng Mobile App thế hệ mới (Microservices + Hybrid Cloud): Tăng hiệu năng, khả năng mở rộng, góp phần nâng tỷ lệ giao dịch số lên 78%.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=36</v>
       </c>
     </row>
     <row r="56" hidden="1">
@@ -15984,7 +15978,7 @@
         <v>1</v>
       </c>
       <c r="F56" t="s">
-        <v>1162</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="57" hidden="1">
@@ -16004,7 +15998,7 @@
         <v>2</v>
       </c>
       <c r="F57" t="s">
-        <v>1163</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="58" hidden="1">
@@ -16027,7 +16021,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="59" hidden="1">
+    <row r="59" ht="350" hidden="1" customHeight="1">
       <c r="A59" t="s">
         <v>364</v>
       </c>
@@ -16043,8 +16037,14 @@
       <c r="E59">
         <v>3</v>
       </c>
-      <c r="F59" t="s">
-        <v>1164</v>
+      <c r="F59" s="2" t="str">
+        <v>BCTN 2025 ghi nhận chuẩn hóa văn bản pháp lý thành quy trình đánh giá tác động hệ thống và trên 90% yêu cầu được cấu hình hóa vào hệ thống công nghệ thông tin. BCTN 2024 ghi nhận các lựa chọn iName và tài khoản số đẹp trên kênh số.
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Chuẩn hóa 100% văn bản pháp lý thành quy trình đánh giá tác động hệ thống, trên 90% yêu cầu được cấu hình hóa vào hệ thống công nghệ thông tin.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=35
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 25 (trang in 48–49)
+Trích đoạn: “Hơn 1 triệu Khách hàng đăng ký mới app LPBank, 86 tính năng sản phẩm mới được triển khai”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=25</v>
       </c>
     </row>
     <row r="60" hidden="1">
@@ -16064,7 +16064,7 @@
         <v>1</v>
       </c>
       <c r="F60" t="s">
-        <v>1165</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="61" hidden="1">
@@ -16084,7 +16084,7 @@
         <v>3</v>
       </c>
       <c r="F61" t="s">
-        <v>1166</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="62" hidden="1">
@@ -16104,7 +16104,7 @@
         <v>1</v>
       </c>
       <c r="F62" t="s">
-        <v>1167</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="63" hidden="1">
@@ -16124,10 +16124,10 @@
         <v>2</v>
       </c>
       <c r="F63" t="s">
-        <v>1168</v>
-      </c>
-    </row>
-    <row r="64" hidden="1">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="64" ht="238" hidden="1" customHeight="1">
       <c r="A64" t="s">
         <v>364</v>
       </c>
@@ -16143,8 +16143,11 @@
       <c r="E64">
         <v>3</v>
       </c>
-      <c r="F64" t="s">
-        <v>1169</v>
+      <c r="F64" s="2" t="str">
+        <v>BCTN 2024 ghi nhận cài đặt phần mềm dò quét mã độc trên các hệ thống dịch vụ quan trọng như Ebanking, LPBank Biz, Core Banking, App LPBank, AD và LIM. Phần mềm được sử dụng để rà quét, xử lý dấu hiệu vi phạm và hỗ trợ điều tra, truy vết; ngân hàng đồng thời nâng cấp bảo mật Data Center và Forcepoint V5000.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Triển khai cài đặt phần mềm dò quét trên các hệ thống dịch vụ đặc biệt quan trọng, có nguy cơ gây thất thoát tiền hoặc thông tin”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=35</v>
       </c>
     </row>
     <row r="65" hidden="1">
@@ -16164,7 +16167,7 @@
         <v>3</v>
       </c>
       <c r="F65" t="s">
-        <v>1170</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="66" hidden="1">
@@ -16184,10 +16187,10 @@
         <v>2</v>
       </c>
       <c r="F66" t="s">
-        <v>1171</v>
-      </c>
-    </row>
-    <row r="67" hidden="1">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="67" ht="364" hidden="1" customHeight="1">
       <c r="A67" t="s">
         <v>364</v>
       </c>
@@ -16203,8 +16206,14 @@
       <c r="E67">
         <v>3</v>
       </c>
-      <c r="F67" t="s">
-        <v>1172</v>
+      <c r="F67" s="2" t="str">
+        <v>BCTN 2025 ghi nhận AI dự báo khách hàng ngừng sử dụng sản phẩm, AI cảnh báo sớm nợ xấu, AI dự báo dòng tiền ALM, AI Chatbot/trợ lý ảo LITA 24/7 và học máy phân tích hành vi. Các dự án gắn với nền tảng dữ liệu và chương trình chuyển đổi số công bố cho năm 2025.
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 36 (trang in 70–71)
+Trích đoạn: “Nâng cấp nền tảng Mobile App thế hệ mới (Microservices + Hybrid Cloud): Tăng hiệu năng, khả năng mở rộng, góp phần nâng tỷ lệ giao dịch số lên 78%.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=36
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Năm 2025, Khối Công nghệ Thông tin đã vận hành mô hình quản trị dự án tập trung để điều phối toàn bộ dự án chuyển đổi số.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=35</v>
       </c>
     </row>
     <row r="68" hidden="1">
@@ -16224,7 +16233,7 @@
         <v>4</v>
       </c>
       <c r="F68" t="s">
-        <v>1173</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="69" hidden="1">
@@ -16244,7 +16253,7 @@
         <v>3</v>
       </c>
       <c r="F69" t="s">
-        <v>1174</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="70" hidden="1">
@@ -16264,7 +16273,7 @@
         <v>3</v>
       </c>
       <c r="F70" t="s">
-        <v>1175</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="71" hidden="1">
@@ -16284,7 +16293,7 @@
         <v>0</v>
       </c>
       <c r="F71" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="72" hidden="1">
@@ -16304,7 +16313,7 @@
         <v>3</v>
       </c>
       <c r="F72" t="s">
-        <v>1177</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="73" hidden="1">
@@ -16324,7 +16333,7 @@
         <v>3</v>
       </c>
       <c r="F73" t="s">
-        <v>1178</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="74" hidden="1">
@@ -16344,7 +16353,7 @@
         <v>2</v>
       </c>
       <c r="F74" t="s">
-        <v>1179</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="75" hidden="1">
@@ -16364,7 +16373,7 @@
         <v>3</v>
       </c>
       <c r="F75" t="s">
-        <v>1180</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="76" hidden="1">
@@ -16387,7 +16396,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="77" hidden="1">
+    <row r="77" ht="364" hidden="1" customHeight="1">
       <c r="A77" t="s">
         <v>364</v>
       </c>
@@ -16403,8 +16412,14 @@
       <c r="E77">
         <v>2</v>
       </c>
-      <c r="F77" t="s">
-        <v>1181</v>
+      <c r="F77" s="2" t="str">
+        <v>BCTN 2025 ghi nhận hoàn thiện hạ tầng Hybrid Cloud và nâng cấp nền tảng Mobile App thế hệ mới theo Microservices + Hybrid Cloud để tăng hiệu năng, khả năng mở rộng. Các nội dung được báo cáo trong chương trình chuyển đổi số và dự án công nghệ năm 2025.
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 36 (trang in 70–71)
+Trích đoạn: “Nâng cấp nền tảng Mobile App thế hệ mới (Microservices + Hybrid Cloud): Tăng hiệu năng, khả năng mở rộng, góp phần nâng tỷ lệ giao dịch số lên 78%.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=36
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Năm 2025, Khối Công nghệ Thông tin đã vận hành mô hình quản trị dự án tập trung để điều phối toàn bộ dự án chuyển đổi số.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=35</v>
       </c>
     </row>
     <row r="78" hidden="1">
@@ -16424,7 +16439,7 @@
         <v>0</v>
       </c>
       <c r="F78" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="79" hidden="1">
@@ -16444,7 +16459,7 @@
         <v>3</v>
       </c>
       <c r="F79" t="s">
-        <v>1182</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="80" hidden="1">
@@ -16484,7 +16499,7 @@
         <v>3</v>
       </c>
       <c r="F81" t="s">
-        <v>1183</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="82" hidden="1">
@@ -16504,7 +16519,7 @@
         <v>3</v>
       </c>
       <c r="F82" t="s">
-        <v>1184</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="83" hidden="1">
@@ -16524,7 +16539,7 @@
         <v>3</v>
       </c>
       <c r="F83" t="s">
-        <v>1185</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="84" hidden="1">
@@ -16547,7 +16562,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="85" hidden="1">
+    <row r="85" ht="336" hidden="1" customHeight="1">
       <c r="A85" t="s">
         <v>573</v>
       </c>
@@ -16563,8 +16578,14 @@
       <c r="E85">
         <v>3</v>
       </c>
-      <c r="F85" t="s">
-        <v>1186</v>
+      <c r="F85" s="2" t="str">
+        <v>BCTN 2024 mô tả dự án UI/UX tối ưu giao diện ứng dụng nhằm nâng cao trải nghiệm khách hàng. BCTN 2025 nêu việc thiết kế sản phẩm, mô hình phục vụ, vận hành và trải nghiệm dựa trên hành trình khách hàng ở cả kênh số và kênh vật lý.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 34 (trang in 66–67)
+Trích đoạn: “Dự án UI/UX: Tối ưu giao diện sản phẩm nhằm nâng cao trải nghiệm Khách hàng trên kênh ứng dụng ngân hàng số LPBank.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=34
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 26 (trang in 50–51)
+Trích đoạn: “Sản phẩm, chính sách, mô hình phục vụ, mô hình vận hành và trải nghiệm được thiết kế dựa trên hành trình khách hàng”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=26</v>
       </c>
     </row>
     <row r="86" hidden="1">
@@ -16584,7 +16605,7 @@
         <v>2</v>
       </c>
       <c r="F86" t="s">
-        <v>1187</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="87" hidden="1">
@@ -16607,7 +16628,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="88" hidden="1">
+    <row r="88" ht="409" hidden="1" customHeight="1">
       <c r="A88" t="s">
         <v>573</v>
       </c>
@@ -16623,8 +16644,17 @@
       <c r="E88">
         <v>3</v>
       </c>
-      <c r="F88" t="s">
-        <v>1188</v>
+      <c r="F88" s="2" t="str">
+        <v>Trong năm 2024, LPBank triển khai 86 tính năng/sản phẩm mới, cải tiến giao diện ứng dụng và ra mắt LPBank Biz. BCTN 2025 tiếp tục mô tả phát triển giải pháp theo phân khúc, combo sản phẩm và mô hình LPBank Priority, gắn với nhu cầu và vòng đời khách hàng.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 25 (trang in 48–49)
+Trích đoạn: “Hơn 1 triệu Khách hàng đăng ký mới app LPBank, 86 tính năng sản phẩm mới được triển khai”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=25
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 32 (trang in 62–63)
+Trích đoạn: “Sau thời gian triển khai chỉ 7 tháng, LPBank đã đưa vào hoạt động ổn định giải pháp ngân hàng lõi CoreBanking T24.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=32
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 27 (trang in 52–53)
+Trích đoạn: “Thiết kế giải pháp theo phân khúc. Ưu tiên giải pháp Combo để một điểm chạm khách hàng được dùng nhiều sản phẩm”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=27</v>
       </c>
     </row>
     <row r="89" hidden="1">
@@ -16644,7 +16674,7 @@
         <v>3</v>
       </c>
       <c r="F89" t="s">
-        <v>1189</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="90" hidden="1">
@@ -16664,10 +16694,10 @@
         <v>3</v>
       </c>
       <c r="F90" t="s">
-        <v>1190</v>
-      </c>
-    </row>
-    <row r="91" hidden="1">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="91" ht="350" hidden="1" customHeight="1">
       <c r="A91" t="s">
         <v>573</v>
       </c>
@@ -16683,8 +16713,14 @@
       <c r="E91">
         <v>3</v>
       </c>
-      <c r="F91" t="s">
-        <v>1191</v>
+      <c r="F91" s="2" t="str">
+        <v>BCTN 2024 ghi nhận quy trình chuyển đổi CoreBanking T24 được kiểm soát chặt chẽ và hệ thống được đưa vào hoạt động ổn định sau 7 tháng triển khai. Năm 2025, LPBank công bố mô hình quản trị dự án tập trung và tỷ lệ dự án hoàn thành go-live, đúng tiến độ là 88%.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 32 (trang in 62–63)
+Trích đoạn: “Sau thời gian triển khai chỉ 7 tháng, LPBank đã đưa vào hoạt động ổn định giải pháp ngân hàng lõi CoreBanking T24.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=32
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Năm 2025, Khối Công nghệ Thông tin đã vận hành mô hình quản trị dự án tập trung để điều phối toàn bộ dự án chuyển đổi số.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=35</v>
       </c>
     </row>
     <row r="92" hidden="1">
@@ -16744,7 +16780,7 @@
         <v>3</v>
       </c>
       <c r="F94" t="s">
-        <v>1192</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="95" hidden="1">
@@ -16764,7 +16800,7 @@
         <v>0</v>
       </c>
       <c r="F95" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="96" hidden="1">
@@ -16784,7 +16820,7 @@
         <v>0</v>
       </c>
       <c r="F96" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="97" hidden="1">
@@ -16804,7 +16840,7 @@
         <v>3</v>
       </c>
       <c r="F97" t="s">
-        <v>1193</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="98" hidden="1">
@@ -16824,7 +16860,7 @@
         <v>3</v>
       </c>
       <c r="F98" t="s">
-        <v>1194</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="99" hidden="1">
@@ -16844,10 +16880,10 @@
         <v>3</v>
       </c>
       <c r="F99" t="s">
-        <v>1195</v>
-      </c>
-    </row>
-    <row r="100" hidden="1">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="100" ht="409" hidden="1" customHeight="1">
       <c r="A100" t="s">
         <v>573</v>
       </c>
@@ -16863,11 +16899,20 @@
       <c r="E100">
         <v>3</v>
       </c>
-      <c r="F100" t="s">
-        <v>1196</v>
-      </c>
-    </row>
-    <row r="101" hidden="1">
+      <c r="F100" s="2" t="str">
+        <v>LPBank triển khai sinh trắc học từ 01/07/2024, phần mềm dò quét mã độc trên các hệ thống dịch vụ quan trọng và các dự án quản lý rủi ro được mô tả trong BCTN 2024. BCTN 2025 ghi nhận các dự án AI cảnh báo rủi ro, học máy phân tích hành vi và nâng cấp bảo mật theo ISO/IEC 27001, PCI-DSS.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 34 (trang in 66–67)
+Trích đoạn: “Dự án UI/UX: Tối ưu giao diện sản phẩm nhằm nâng cao trải nghiệm Khách hàng trên kênh ứng dụng ngân hàng số LPBank.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=34
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Triển khai cài đặt phần mềm dò quét trên các hệ thống dịch vụ đặc biệt quan trọng, có nguy cơ gây thất thoát tiền hoặc thông tin”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=35
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 36 (trang in 70–71)
+Trích đoạn: “Nâng cấp nền tảng Mobile App thế hệ mới (Microservices + Hybrid Cloud): Tăng hiệu năng, khả năng mở rộng, góp phần nâng tỷ lệ giao dịch số lên 78%.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=36</v>
+      </c>
+    </row>
+    <row r="101" ht="364" hidden="1" customHeight="1">
       <c r="A101" t="s">
         <v>573</v>
       </c>
@@ -16883,8 +16928,14 @@
       <c r="E101">
         <v>3</v>
       </c>
-      <c r="F101" t="s">
-        <v>1197</v>
+      <c r="F101" s="2" t="str">
+        <v>BCTN 2024 ghi nhận CoreBanking T24 đi vào hoạt động ổn định và Kondor Treasury được đưa vào vận hành. BCTN 2025 mô tả mô hình DC1–DC2–DR Active–Active và nâng cấp Mobile App theo Microservices + Hybrid Cloud để phục vụ vận hành liên tục, tăng hiệu năng và khả năng mở rộng.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 32 (trang in 62–63)
+Trích đoạn: “Sau thời gian triển khai chỉ 7 tháng, LPBank đã đưa vào hoạt động ổn định giải pháp ngân hàng lõi CoreBanking T24.”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=32
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 36 (trang in 70–71)
+Trích đoạn: “Nâng cấp nền tảng Mobile App thế hệ mới (Microservices + Hybrid Cloud): Tăng hiệu năng, khả năng mở rộng, góp phần nâng tỷ lệ giao dịch số lên 78%.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=36</v>
       </c>
     </row>
     <row r="102" hidden="1">
@@ -17004,7 +17055,7 @@
         <v>3</v>
       </c>
       <c r="F107" t="s">
-        <v>1198</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="108" hidden="1">
@@ -17024,7 +17075,7 @@
         <v>3</v>
       </c>
       <c r="F108" t="s">
-        <v>1199</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="109" hidden="1">
@@ -17044,7 +17095,7 @@
         <v>3</v>
       </c>
       <c r="F109" t="s">
-        <v>1200</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="110" hidden="1">
@@ -17064,7 +17115,7 @@
         <v>1</v>
       </c>
       <c r="F110" t="s">
-        <v>1201</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="111" hidden="1">
@@ -17084,7 +17135,7 @@
         <v>0</v>
       </c>
       <c r="F111" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="112" hidden="1">
@@ -17104,7 +17155,7 @@
         <v>3</v>
       </c>
       <c r="F112" t="s">
-        <v>1202</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="113" hidden="1">
@@ -17124,7 +17175,7 @@
         <v>3</v>
       </c>
       <c r="F113" t="s">
-        <v>1203</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="114" hidden="1">
@@ -17144,7 +17195,7 @@
         <v>3</v>
       </c>
       <c r="F114" t="s">
-        <v>1204</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="115" hidden="1">
@@ -17164,7 +17215,7 @@
         <v>0</v>
       </c>
       <c r="F115" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="116" hidden="1">
@@ -17184,7 +17235,7 @@
         <v>0</v>
       </c>
       <c r="F116" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="117" hidden="1">
@@ -17204,7 +17255,7 @@
         <v>0</v>
       </c>
       <c r="F117" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="118" hidden="1">
@@ -17224,7 +17275,7 @@
         <v>0</v>
       </c>
       <c r="F118" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="119" hidden="1">
@@ -17244,7 +17295,7 @@
         <v>0</v>
       </c>
       <c r="F119" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="120" hidden="1">
@@ -17264,7 +17315,7 @@
         <v>3</v>
       </c>
       <c r="F120" t="s">
-        <v>1205</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="121" hidden="1">
@@ -17284,7 +17335,7 @@
         <v>3</v>
       </c>
       <c r="F121" t="s">
-        <v>1206</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="122" hidden="1">
@@ -17304,7 +17355,7 @@
         <v>0</v>
       </c>
       <c r="F122" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="123" hidden="1">
@@ -17324,7 +17375,7 @@
         <v>3</v>
       </c>
       <c r="F123" t="s">
-        <v>1207</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="124">
@@ -17344,7 +17395,7 @@
         <v>0</v>
       </c>
       <c r="F124" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="125">
@@ -17364,7 +17415,7 @@
         <v>3</v>
       </c>
       <c r="F125" t="s">
-        <v>1208</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="126">
@@ -17384,10 +17435,10 @@
         <v>0</v>
       </c>
       <c r="F126" t="s">
-        <v>1176</v>
-      </c>
-    </row>
-    <row r="127">
+        <v>1160</v>
+      </c>
+    </row>
+    <row r="127" ht="364" customHeight="1">
       <c r="A127" t="s">
         <v>890</v>
       </c>
@@ -17403,8 +17454,14 @@
       <c r="E127">
         <v>3</v>
       </c>
-      <c r="F127" t="s">
-        <v>1209</v>
+      <c r="F127" s="2" t="str">
+        <v>BCTN 2024 ghi nhận dò quét mã độc trên hệ thống giao dịch, xác thực và ứng dụng; đầu tư bảo mật Data Center và nâng cấp Forcepoint V5000. BCTN 2025 ghi nhận triển khai ISO/IEC 27001 và nâng cấp bảo mật đạt chuẩn PCI-DSS trong chương trình công nghệ của năm.
+Nguồn: Báo cáo thường niên LP Bank 2024 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Triển khai cài đặt phần mềm dò quét trên các hệ thống dịch vụ đặc biệt quan trọng, có nguy cơ gây thất thoát tiền hoặc thông tin”
+https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=35
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 36 (trang in 70–71)
+Trích đoạn: “Nâng cấp nền tảng Mobile App thế hệ mới (Microservices + Hybrid Cloud): Tăng hiệu năng, khả năng mở rộng, góp phần nâng tỷ lệ giao dịch số lên 78%.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=36</v>
       </c>
     </row>
     <row r="128">
@@ -17424,7 +17481,7 @@
         <v>3</v>
       </c>
       <c r="F128" t="s">
-        <v>1210</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="129">
@@ -17444,7 +17501,7 @@
         <v>0</v>
       </c>
       <c r="F129" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="130">
@@ -17464,7 +17521,7 @@
         <v>0</v>
       </c>
       <c r="F130" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="131">
@@ -17484,7 +17541,7 @@
         <v>3</v>
       </c>
       <c r="F131" t="s">
-        <v>1211</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="132">
@@ -17504,7 +17561,7 @@
         <v>0</v>
       </c>
       <c r="F132" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="133">
@@ -17524,7 +17581,7 @@
         <v>3</v>
       </c>
       <c r="F133" t="s">
-        <v>1212</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="134">
@@ -17544,7 +17601,7 @@
         <v>3</v>
       </c>
       <c r="F134" t="s">
-        <v>1213</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="135">
@@ -17564,7 +17621,7 @@
         <v>0</v>
       </c>
       <c r="F135" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="136">
@@ -17584,7 +17641,7 @@
         <v>3</v>
       </c>
       <c r="F136" t="s">
-        <v>1214</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="137">
@@ -17604,7 +17661,7 @@
         <v>0</v>
       </c>
       <c r="F137" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="138">
@@ -17624,7 +17681,7 @@
         <v>3</v>
       </c>
       <c r="F138" t="s">
-        <v>1215</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="139">
@@ -17644,10 +17701,10 @@
         <v>3</v>
       </c>
       <c r="F139" t="s">
-        <v>1216</v>
-      </c>
-    </row>
-    <row r="140">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="140" ht="378" customHeight="1">
       <c r="A140" t="s">
         <v>890</v>
       </c>
@@ -17663,8 +17720,14 @@
       <c r="E140">
         <v>3</v>
       </c>
-      <c r="F140" t="s">
-        <v>1217</v>
+      <c r="F140" s="2" t="str">
+        <v>BCTN 2025 ghi nhận nền tảng Data Lakehouse, Customer 360/CDP và các ứng dụng AI/ML: dự báo khách hàng ngừng sử dụng sản phẩm, cảnh báo sớm nợ xấu, dự báo dòng tiền ALM, chatbot/trợ lý ảo LITA và phân tích hành vi. Đây là các ứng dụng khai thác dữ liệu được ngân hàng công bố trong năm 2025.
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 35 (trang in 68–69)
+Trích đoạn: “Năm 2025, Khối Công nghệ Thông tin đã vận hành mô hình quản trị dự án tập trung để điều phối toàn bộ dự án chuyển đổi số.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=35
+Nguồn: Báo cáo thường niên LP Bank 2025 · trang PDF 36 (trang in 70–71)
+Trích đoạn: “Nâng cấp nền tảng Mobile App thế hệ mới (Microservices + Hybrid Cloud): Tăng hiệu năng, khả năng mở rộng, góp phần nâng tỷ lệ giao dịch số lên 78%.”
+https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=36</v>
       </c>
     </row>
     <row r="141">
@@ -17684,7 +17747,7 @@
         <v>0</v>
       </c>
       <c r="F141" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
   </sheetData>
@@ -17836,7 +17899,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>1218</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="7" hidden="1">
@@ -17880,7 +17943,7 @@
         <v>3</v>
       </c>
       <c r="F8" t="s">
-        <v>1219</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="9" hidden="1">
@@ -17900,7 +17963,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="s">
-        <v>1220</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="10" hidden="1">
@@ -17920,7 +17983,7 @@
         <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>1221</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="11" hidden="1">
@@ -17940,7 +18003,7 @@
         <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>1222</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="12" hidden="1">
@@ -17960,7 +18023,7 @@
         <v>3</v>
       </c>
       <c r="F12" t="s">
-        <v>1223</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="13" hidden="1">
@@ -17980,7 +18043,7 @@
         <v>2</v>
       </c>
       <c r="F13" t="s">
-        <v>1224</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="14" hidden="1">
@@ -18000,7 +18063,7 @@
         <v>4</v>
       </c>
       <c r="F14" t="s">
-        <v>1225</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="15" hidden="1">
@@ -18020,7 +18083,7 @@
         <v>4</v>
       </c>
       <c r="F15" t="s">
-        <v>1226</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="16" hidden="1">
@@ -18040,7 +18103,7 @@
         <v>3</v>
       </c>
       <c r="F16" t="s">
-        <v>1227</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="17" hidden="1">
@@ -18060,7 +18123,7 @@
         <v>4</v>
       </c>
       <c r="F17" t="s">
-        <v>1228</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="18" hidden="1">
@@ -18080,7 +18143,7 @@
         <v>3</v>
       </c>
       <c r="F18" t="s">
-        <v>1229</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="19" hidden="1">
@@ -18100,7 +18163,7 @@
         <v>2</v>
       </c>
       <c r="F19" t="s">
-        <v>1230</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="20" hidden="1">
@@ -18120,7 +18183,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="s">
-        <v>1231</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="21" hidden="1">
@@ -18140,7 +18203,7 @@
         <v>3</v>
       </c>
       <c r="F21" t="s">
-        <v>1232</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="22" hidden="1">
@@ -18160,7 +18223,7 @@
         <v>4</v>
       </c>
       <c r="F22" t="s">
-        <v>1233</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="23" hidden="1">
@@ -18180,7 +18243,7 @@
         <v>4</v>
       </c>
       <c r="F23" t="s">
-        <v>1234</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="24" hidden="1">
@@ -18200,7 +18263,7 @@
         <v>4</v>
       </c>
       <c r="F24" t="s">
-        <v>1235</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="25" hidden="1">
@@ -18220,7 +18283,7 @@
         <v>4</v>
       </c>
       <c r="F25" t="s">
-        <v>1236</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="26" hidden="1">
@@ -18240,7 +18303,7 @@
         <v>3</v>
       </c>
       <c r="F26" t="s">
-        <v>1237</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="27" hidden="1">
@@ -18348,7 +18411,7 @@
         <v>4</v>
       </c>
       <c r="F31" t="s">
-        <v>1238</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="32" hidden="1">
@@ -18368,7 +18431,7 @@
         <v>4</v>
       </c>
       <c r="F32" t="s">
-        <v>1239</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="33" hidden="1">
@@ -18388,7 +18451,7 @@
         <v>4</v>
       </c>
       <c r="F33" t="s">
-        <v>1240</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="34" hidden="1">
@@ -18408,7 +18471,7 @@
         <v>3</v>
       </c>
       <c r="F34" t="s">
-        <v>1241</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="35" hidden="1">
@@ -18428,7 +18491,7 @@
         <v>0</v>
       </c>
       <c r="F35" t="s">
-        <v>1242</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="36" hidden="1">
@@ -18448,7 +18511,7 @@
         <v>3</v>
       </c>
       <c r="F36" t="s">
-        <v>1243</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="37" hidden="1">
@@ -18468,7 +18531,7 @@
         <v>3</v>
       </c>
       <c r="F37" t="s">
-        <v>1244</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="38" hidden="1">
@@ -18488,7 +18551,7 @@
         <v>3</v>
       </c>
       <c r="F38" t="s">
-        <v>1245</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="39" hidden="1">
@@ -18508,7 +18571,7 @@
         <v>3</v>
       </c>
       <c r="F39" t="s">
-        <v>1246</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="40" hidden="1">
@@ -18528,7 +18591,7 @@
         <v>4</v>
       </c>
       <c r="F40" t="s">
-        <v>1247</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="41" hidden="1">
@@ -18548,7 +18611,7 @@
         <v>3</v>
       </c>
       <c r="F41" t="s">
-        <v>1248</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="42" hidden="1">
@@ -18568,7 +18631,7 @@
         <v>4</v>
       </c>
       <c r="F42" t="s">
-        <v>1249</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="43" hidden="1">
@@ -18588,7 +18651,7 @@
         <v>4</v>
       </c>
       <c r="F43" t="s">
-        <v>1250</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="44" hidden="1">
@@ -18608,7 +18671,7 @@
         <v>3</v>
       </c>
       <c r="F44" t="s">
-        <v>1251</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="45" hidden="1">
@@ -18628,7 +18691,7 @@
         <v>4</v>
       </c>
       <c r="F45" t="s">
-        <v>1252</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="46" hidden="1">
@@ -18648,7 +18711,7 @@
         <v>4</v>
       </c>
       <c r="F46" t="s">
-        <v>1253</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="47" hidden="1">
@@ -18668,7 +18731,7 @@
         <v>3</v>
       </c>
       <c r="F47" t="s">
-        <v>1254</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="48" hidden="1">
@@ -18688,7 +18751,7 @@
         <v>4</v>
       </c>
       <c r="F48" t="s">
-        <v>1255</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -18708,7 +18771,7 @@
         <v>3</v>
       </c>
       <c r="F49" t="s">
-        <v>1256</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -18728,7 +18791,7 @@
         <v>0</v>
       </c>
       <c r="F50" t="s">
-        <v>1257</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -18748,7 +18811,7 @@
         <v>3</v>
       </c>
       <c r="F51" t="s">
-        <v>1258</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -18768,7 +18831,7 @@
         <v>4</v>
       </c>
       <c r="F52" t="s">
-        <v>1259</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="53" hidden="1">
@@ -18788,7 +18851,7 @@
         <v>3</v>
       </c>
       <c r="F53" t="s">
-        <v>1260</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="54" hidden="1">
@@ -18808,7 +18871,7 @@
         <v>3</v>
       </c>
       <c r="F54" t="s">
-        <v>1261</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="55" hidden="1">
@@ -18828,7 +18891,7 @@
         <v>4</v>
       </c>
       <c r="F55" t="s">
-        <v>1262</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="56" hidden="1">
@@ -18848,7 +18911,7 @@
         <v>3</v>
       </c>
       <c r="F56" t="s">
-        <v>1263</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="57" hidden="1">
@@ -18868,7 +18931,7 @@
         <v>0</v>
       </c>
       <c r="F57" t="s">
-        <v>1264</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="58" hidden="1">
@@ -18888,7 +18951,7 @@
         <v>0</v>
       </c>
       <c r="F58" t="s">
-        <v>1265</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="59" hidden="1">
@@ -18908,7 +18971,7 @@
         <v>3</v>
       </c>
       <c r="F59" t="s">
-        <v>1266</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="60" hidden="1">
@@ -18928,7 +18991,7 @@
         <v>4</v>
       </c>
       <c r="F60" t="s">
-        <v>1267</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="61" hidden="1">
@@ -18948,7 +19011,7 @@
         <v>4</v>
       </c>
       <c r="F61" t="s">
-        <v>1268</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="62" hidden="1">
@@ -18968,7 +19031,7 @@
         <v>3</v>
       </c>
       <c r="F62" t="s">
-        <v>1269</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="63" hidden="1">
@@ -18988,7 +19051,7 @@
         <v>4</v>
       </c>
       <c r="F63" t="s">
-        <v>1270</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="64" hidden="1">
@@ -19008,7 +19071,7 @@
         <v>4</v>
       </c>
       <c r="F64" t="s">
-        <v>1271</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="65" hidden="1">
@@ -19028,7 +19091,7 @@
         <v>4</v>
       </c>
       <c r="F65" t="s">
-        <v>1272</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="66" hidden="1">
@@ -19048,7 +19111,7 @@
         <v>0</v>
       </c>
       <c r="F66" t="s">
-        <v>1273</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="67" hidden="1">
@@ -19068,7 +19131,7 @@
         <v>3</v>
       </c>
       <c r="F67" t="s">
-        <v>1274</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="68" hidden="1">
@@ -19088,7 +19151,7 @@
         <v>3</v>
       </c>
       <c r="F68" t="s">
-        <v>1275</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="69" hidden="1">
@@ -19108,7 +19171,7 @@
         <v>3</v>
       </c>
       <c r="F69" t="s">
-        <v>1276</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="70" hidden="1">
@@ -19128,7 +19191,7 @@
         <v>3</v>
       </c>
       <c r="F70" t="s">
-        <v>1277</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="71" hidden="1">
@@ -19148,7 +19211,7 @@
         <v>0</v>
       </c>
       <c r="F71" t="s">
-        <v>1278</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="72" hidden="1">
@@ -19168,7 +19231,7 @@
         <v>3</v>
       </c>
       <c r="F72" t="s">
-        <v>1279</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="73" hidden="1">
@@ -19188,7 +19251,7 @@
         <v>2</v>
       </c>
       <c r="F73" t="s">
-        <v>1280</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="74" hidden="1">
@@ -19208,7 +19271,7 @@
         <v>0</v>
       </c>
       <c r="F74" t="s">
-        <v>1281</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="75" hidden="1">
@@ -19228,7 +19291,7 @@
         <v>3</v>
       </c>
       <c r="F75" t="s">
-        <v>1282</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="76" hidden="1">
@@ -19248,7 +19311,7 @@
         <v>2</v>
       </c>
       <c r="F76" t="s">
-        <v>1283</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="77" hidden="1">
@@ -19268,7 +19331,7 @@
         <v>4</v>
       </c>
       <c r="F77" t="s">
-        <v>1284</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="78" hidden="1">
@@ -19288,7 +19351,7 @@
         <v>0</v>
       </c>
       <c r="F78" t="s">
-        <v>1285</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="79" hidden="1">
@@ -19308,7 +19371,7 @@
         <v>4</v>
       </c>
       <c r="F79" t="s">
-        <v>1286</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="80" hidden="1">
@@ -19328,7 +19391,7 @@
         <v>3</v>
       </c>
       <c r="F80" t="s">
-        <v>1287</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="81" hidden="1">
@@ -19348,7 +19411,7 @@
         <v>4</v>
       </c>
       <c r="F81" t="s">
-        <v>1288</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="82" hidden="1">
@@ -19368,7 +19431,7 @@
         <v>4</v>
       </c>
       <c r="F82" t="s">
-        <v>1289</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="83" hidden="1">
@@ -19388,7 +19451,7 @@
         <v>0</v>
       </c>
       <c r="F83" t="s">
-        <v>1290</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="84" hidden="1">
@@ -19408,7 +19471,7 @@
         <v>3</v>
       </c>
       <c r="F84" t="s">
-        <v>1291</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="85" hidden="1">
@@ -19428,7 +19491,7 @@
         <v>0</v>
       </c>
       <c r="F85" t="s">
-        <v>1292</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="86" hidden="1">
@@ -19448,7 +19511,7 @@
         <v>0</v>
       </c>
       <c r="F86" t="s">
-        <v>1293</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="87" hidden="1">
@@ -19468,7 +19531,7 @@
         <v>4</v>
       </c>
       <c r="F87" t="s">
-        <v>1294</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="88" hidden="1">
@@ -19488,7 +19551,7 @@
         <v>4</v>
       </c>
       <c r="F88" t="s">
-        <v>1295</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="89" hidden="1">
@@ -19508,7 +19571,7 @@
         <v>4</v>
       </c>
       <c r="F89" t="s">
-        <v>1296</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="90" hidden="1">
@@ -19528,7 +19591,7 @@
         <v>2</v>
       </c>
       <c r="F90" t="s">
-        <v>1297</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="91" hidden="1">
@@ -19548,7 +19611,7 @@
         <v>2</v>
       </c>
       <c r="F91" t="s">
-        <v>1298</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="92" hidden="1">
@@ -19568,7 +19631,7 @@
         <v>4</v>
       </c>
       <c r="F92" t="s">
-        <v>1299</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="93" hidden="1">
@@ -19588,7 +19651,7 @@
         <v>0</v>
       </c>
       <c r="F93" t="s">
-        <v>1300</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="94" hidden="1">
@@ -19608,7 +19671,7 @@
         <v>4</v>
       </c>
       <c r="F94" t="s">
-        <v>1301</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="95" hidden="1">
@@ -19628,7 +19691,7 @@
         <v>0</v>
       </c>
       <c r="F95" t="s">
-        <v>1302</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="96" hidden="1">
@@ -19648,7 +19711,7 @@
         <v>3</v>
       </c>
       <c r="F96" t="s">
-        <v>1303</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="97" hidden="1">
@@ -19668,7 +19731,7 @@
         <v>4</v>
       </c>
       <c r="F97" t="s">
-        <v>1304</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="98" hidden="1">
@@ -19688,7 +19751,7 @@
         <v>3</v>
       </c>
       <c r="F98" t="s">
-        <v>1305</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="99" hidden="1">
@@ -19708,7 +19771,7 @@
         <v>2</v>
       </c>
       <c r="F99" t="s">
-        <v>1306</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="100" hidden="1">
@@ -19728,7 +19791,7 @@
         <v>4</v>
       </c>
       <c r="F100" t="s">
-        <v>1307</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="101" hidden="1">
@@ -19748,7 +19811,7 @@
         <v>4</v>
       </c>
       <c r="F101" t="s">
-        <v>1308</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="102" hidden="1">
@@ -19768,7 +19831,7 @@
         <v>3</v>
       </c>
       <c r="F102" t="s">
-        <v>1309</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="103" hidden="1">
@@ -19788,7 +19851,7 @@
         <v>3</v>
       </c>
       <c r="F103" t="s">
-        <v>1310</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="104" hidden="1">
@@ -19808,7 +19871,7 @@
         <v>4</v>
       </c>
       <c r="F104" t="s">
-        <v>1311</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="105" hidden="1">
@@ -19828,7 +19891,7 @@
         <v>0</v>
       </c>
       <c r="F105" t="s">
-        <v>1312</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="106" hidden="1">
@@ -19848,7 +19911,7 @@
         <v>0</v>
       </c>
       <c r="F106" t="s">
-        <v>1313</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="107" hidden="1">
@@ -19868,7 +19931,7 @@
         <v>4</v>
       </c>
       <c r="F107" t="s">
-        <v>1314</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="108" hidden="1">
@@ -19888,7 +19951,7 @@
         <v>4</v>
       </c>
       <c r="F108" t="s">
-        <v>1315</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="109" hidden="1">
@@ -19908,7 +19971,7 @@
         <v>4</v>
       </c>
       <c r="F109" t="s">
-        <v>1316</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="110" hidden="1">
@@ -19928,7 +19991,7 @@
         <v>3</v>
       </c>
       <c r="F110" t="s">
-        <v>1317</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="111" hidden="1">
@@ -19948,7 +20011,7 @@
         <v>4</v>
       </c>
       <c r="F111" t="s">
-        <v>1318</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="112" hidden="1">
@@ -19990,7 +20053,7 @@
         <v>4</v>
       </c>
       <c r="F113" t="s">
-        <v>1319</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="114" hidden="1">
@@ -20010,7 +20073,7 @@
         <v>4</v>
       </c>
       <c r="F114" t="s">
-        <v>1320</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="115" hidden="1">
@@ -20030,7 +20093,7 @@
         <v>3</v>
       </c>
       <c r="F115" t="s">
-        <v>1321</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="116" hidden="1">
@@ -20050,7 +20113,7 @@
         <v>3</v>
       </c>
       <c r="F116" t="s">
-        <v>1322</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="117" hidden="1">
@@ -20070,7 +20133,7 @@
         <v>3</v>
       </c>
       <c r="F117" t="s">
-        <v>1323</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="118" hidden="1">
@@ -20090,7 +20153,7 @@
         <v>3</v>
       </c>
       <c r="F118" t="s">
-        <v>1324</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="119" hidden="1">
@@ -20110,7 +20173,7 @@
         <v>3</v>
       </c>
       <c r="F119" t="s">
-        <v>1325</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="120" hidden="1">
@@ -20130,7 +20193,7 @@
         <v>3</v>
       </c>
       <c r="F120" t="s">
-        <v>1326</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="121" hidden="1">
@@ -20150,7 +20213,7 @@
         <v>2</v>
       </c>
       <c r="F121" t="s">
-        <v>1327</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="122" hidden="1">
@@ -20170,7 +20233,7 @@
         <v>3</v>
       </c>
       <c r="F122" t="s">
-        <v>1328</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="123" hidden="1">
@@ -20190,7 +20253,7 @@
         <v>3</v>
       </c>
       <c r="F123" t="s">
-        <v>1329</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="124">
@@ -20210,7 +20273,7 @@
         <v>0</v>
       </c>
       <c r="F124" t="s">
-        <v>1330</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="125">
@@ -20230,7 +20293,7 @@
         <v>3</v>
       </c>
       <c r="F125" t="s">
-        <v>1331</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="126">
@@ -20250,7 +20313,7 @@
         <v>0</v>
       </c>
       <c r="F126" t="s">
-        <v>1332</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="127">
@@ -20270,7 +20333,7 @@
         <v>4</v>
       </c>
       <c r="F127" t="s">
-        <v>1333</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="128">
@@ -20290,7 +20353,7 @@
         <v>4</v>
       </c>
       <c r="F128" t="s">
-        <v>1334</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="129">
@@ -20310,7 +20373,7 @@
         <v>3</v>
       </c>
       <c r="F129" t="s">
-        <v>1335</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="130">
@@ -20330,7 +20393,7 @@
         <v>3</v>
       </c>
       <c r="F130" t="s">
-        <v>1336</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="131">
@@ -20350,7 +20413,7 @@
         <v>4</v>
       </c>
       <c r="F131" t="s">
-        <v>1337</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="132">
@@ -20370,7 +20433,7 @@
         <v>4</v>
       </c>
       <c r="F132" t="s">
-        <v>1338</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="133">
@@ -20390,7 +20453,7 @@
         <v>4</v>
       </c>
       <c r="F133" t="s">
-        <v>1339</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="134">
@@ -20410,7 +20473,7 @@
         <v>3</v>
       </c>
       <c r="F134" t="s">
-        <v>1340</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="135">
@@ -20430,7 +20493,7 @@
         <v>0</v>
       </c>
       <c r="F135" t="s">
-        <v>1341</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="136">
@@ -20450,7 +20513,7 @@
         <v>3</v>
       </c>
       <c r="F136" t="s">
-        <v>1342</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="137">
@@ -20470,7 +20533,7 @@
         <v>2</v>
       </c>
       <c r="F137" t="s">
-        <v>1343</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="138">
@@ -20490,7 +20553,7 @@
         <v>0</v>
       </c>
       <c r="F138" t="s">
-        <v>1344</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="139">
@@ -20510,7 +20573,7 @@
         <v>3</v>
       </c>
       <c r="F139" t="s">
-        <v>1345</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="140">
@@ -20530,7 +20593,7 @@
         <v>3</v>
       </c>
       <c r="F140" t="s">
-        <v>1346</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="141">
@@ -20550,7 +20613,7 @@
         <v>2</v>
       </c>
       <c r="F141" t="s">
-        <v>1347</v>
+        <v>1323</v>
       </c>
     </row>
   </sheetData>
@@ -20614,7 +20677,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>1348</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="3" hidden="1">
@@ -20634,7 +20697,7 @@
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>1349</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="4" hidden="1">
@@ -20654,7 +20717,7 @@
         <v>2</v>
       </c>
       <c r="F4" t="s">
-        <v>1350</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="5" hidden="1">
@@ -20674,7 +20737,7 @@
         <v>2</v>
       </c>
       <c r="F5" t="s">
-        <v>1351</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="6" hidden="1">
@@ -20694,7 +20757,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>1352</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="7" hidden="1">
@@ -20714,7 +20777,7 @@
         <v>2</v>
       </c>
       <c r="F7" t="s">
-        <v>1353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="8" hidden="1">
@@ -20734,7 +20797,7 @@
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>1354</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="9" hidden="1">
@@ -20754,7 +20817,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="s">
-        <v>1355</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="10" hidden="1">
@@ -20774,7 +20837,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="s">
-        <v>1356</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="11" hidden="1">
@@ -20794,7 +20857,7 @@
         <v>2</v>
       </c>
       <c r="F11" t="s">
-        <v>1357</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="12" hidden="1">
@@ -20814,7 +20877,7 @@
         <v>2</v>
       </c>
       <c r="F12" t="s">
-        <v>1358</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="13" hidden="1">
@@ -20834,7 +20897,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>1359</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="14" hidden="1">
@@ -20854,7 +20917,7 @@
         <v>2</v>
       </c>
       <c r="F14" t="s">
-        <v>1360</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="15" hidden="1">
@@ -20874,7 +20937,7 @@
         <v>2</v>
       </c>
       <c r="F15" t="s">
-        <v>1361</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="16" hidden="1">
@@ -20894,7 +20957,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>1362</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="17" hidden="1">
@@ -20914,7 +20977,7 @@
         <v>0</v>
       </c>
       <c r="F17" t="s">
-        <v>1363</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="18" hidden="1">
@@ -20934,7 +20997,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="s">
-        <v>1364</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="19" hidden="1">
@@ -20954,7 +21017,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="s">
-        <v>1365</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="20" hidden="1">
@@ -20974,7 +21037,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="s">
-        <v>1366</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="21" hidden="1">
@@ -20994,7 +21057,7 @@
         <v>2</v>
       </c>
       <c r="F21" t="s">
-        <v>1367</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="22" hidden="1">
@@ -21014,7 +21077,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="s">
-        <v>1368</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="23" hidden="1">
@@ -21034,7 +21097,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>1369</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="24" hidden="1">
@@ -21054,7 +21117,7 @@
         <v>3</v>
       </c>
       <c r="F24" t="s">
-        <v>1370</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="25" hidden="1">
@@ -21074,7 +21137,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="s">
-        <v>1371</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="26" hidden="1">
@@ -21094,7 +21157,7 @@
         <v>2</v>
       </c>
       <c r="F26" t="s">
-        <v>1372</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="27">
@@ -21114,7 +21177,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="s">
-        <v>1373</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="28">
@@ -21134,7 +21197,7 @@
         <v>2</v>
       </c>
       <c r="F28" t="s">
-        <v>1374</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="29">
@@ -21154,7 +21217,7 @@
         <v>0</v>
       </c>
       <c r="F29" t="s">
-        <v>1375</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="30">
@@ -21174,7 +21237,7 @@
         <v>2</v>
       </c>
       <c r="F30" t="s">
-        <v>1376</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="31">
@@ -21194,10 +21257,10 @@
         <v>2</v>
       </c>
       <c r="F31" t="s">
-        <v>1377</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>1353</v>
+      </c>
+    </row>
+    <row r="32" ht="280" customHeight="1">
       <c r="A32" t="s">
         <v>189</v>
       </c>
@@ -21213,8 +21276,11 @@
       <c r="E32">
         <v>2</v>
       </c>
-      <c r="F32" t="s">
-        <v>1378</v>
+      <c r="F32" s="2" t="str">
+        <v>Trong kết quả hoạt động năm 2025, SAIGONBANK ghi nhận kết nối tài khoản với VNeID để nhận chi trả an sinh xã hội; triển khai thanh toán không tiếp xúc cho giao thông công cộng, thanh toán tại bãi xe thông minh và tham gia dự án công nghệ hỗ trợ hành chính công. Các nội dung thể hiện các kết nối dịch vụ đã triển khai trong kỳ.
+Nguồn: Báo cáo thường niên SaigonBank 2025 · trang PDF 6 (trang in 5)
+Trích đoạn: “Ngân hàng đã triển khai kết nối tài khoản SAIGONBANK với ứng dụng VNeID của khách hàng liên kết tài khoản SAIGONBANK để nhận chi trả An sinh xã hội qua ứng dụng VNeID”
+https://static2.vietstock.vn/data/HNX/2025/BCTN/VN/SGB_Baocaothuongnien_2025/1_sgb_2026_4_20_43bf2b9_vi_baocaothuongnien_2025_compressedda_ky.pdf#page=6</v>
       </c>
     </row>
     <row r="33">
@@ -21234,7 +21300,7 @@
         <v>0</v>
       </c>
       <c r="F33" t="s">
-        <v>1379</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="34">
@@ -21254,7 +21320,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="s">
-        <v>1380</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="35">
@@ -21274,7 +21340,7 @@
         <v>0</v>
       </c>
       <c r="F35" t="s">
-        <v>1381</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="36">
@@ -21294,7 +21360,7 @@
         <v>0</v>
       </c>
       <c r="F36" t="s">
-        <v>1382</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="37">
@@ -21314,7 +21380,7 @@
         <v>0</v>
       </c>
       <c r="F37" t="s">
-        <v>1383</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="38">
@@ -21334,7 +21400,7 @@
         <v>0</v>
       </c>
       <c r="F38" t="s">
-        <v>1384</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="39">
@@ -21354,7 +21420,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="s">
-        <v>1385</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="40">
@@ -21374,10 +21440,10 @@
         <v>0</v>
       </c>
       <c r="F40" t="s">
-        <v>1386</v>
-      </c>
-    </row>
-    <row r="41">
+        <v>1361</v>
+      </c>
+    </row>
+    <row r="41" ht="406" customHeight="1">
       <c r="A41" t="s">
         <v>189</v>
       </c>
@@ -21393,8 +21459,14 @@
       <c r="E41">
         <v>2</v>
       </c>
-      <c r="F41" t="s">
-        <v>1387</v>
+      <c r="F41" s="2" t="str">
+        <v>BCTN 2024 nêu định hướng hoạt động năm 2025: đẩy mạnh ứng dụng CNTT, thanh toán không dùng tiền mặt và chuyển đổi số theo lộ trình phù hợp. Trong kết quả năm 2025, ngân hàng ghi nhận phát triển tính năng SAIGONBANK PAY/Smart Banking và kết nối VNeID, giao thông công cộng, bãi xe thông minh.
+Nguồn: Báo cáo thường niên SaigonBank 2024 · trang PDF 13 (trang in 12)
+Trích đoạn: “Tập trung đẩy mạnh ứng dụng công nghệ thông tin trong hoạt động ngân hàng và hoạt động thanh toán không dùng tiền mặt”
+https://static2.vietstock.vn/data/HNX/2024/BCTN/VN/SGB_Baocaothuongnien_2024/1_sgb_2025_4_17_56f822a_vi_baocaothuongnien_2024.pdf#page=13
+Nguồn: Báo cáo thường niên SaigonBank 2025 · trang PDF 6 (trang in 5)
+Trích đoạn: “Ngân hàng đã triển khai kết nối tài khoản SAIGONBANK với ứng dụng VNeID của khách hàng liên kết tài khoản SAIGONBANK để nhận chi trả An sinh xã hội qua ứng dụng VNeID”
+https://static2.vietstock.vn/data/HNX/2025/BCTN/VN/SGB_Baocaothuongnien_2025/1_sgb_2026_4_20_43bf2b9_vi_baocaothuongnien_2025_compressedda_ky.pdf#page=6</v>
       </c>
     </row>
     <row r="42">
@@ -21414,10 +21486,10 @@
         <v>2</v>
       </c>
       <c r="F42" t="s">
-        <v>1388</v>
-      </c>
-    </row>
-    <row r="43">
+        <v>1362</v>
+      </c>
+    </row>
+    <row r="43" ht="378" customHeight="1">
       <c r="A43" t="s">
         <v>189</v>
       </c>
@@ -21433,8 +21505,14 @@
       <c r="E43">
         <v>2</v>
       </c>
-      <c r="F43" t="s">
-        <v>1389</v>
+      <c r="F43" s="2" t="str">
+        <v>Trong kết quả hoạt động năm 2024, SAIGONBANK công bố đã hoàn thành xây dựng Chiến lược phát triển đến năm 2025, định hướng đến năm 2030. Định hướng hoạt động năm 2025 trong cùng báo cáo gắn ứng dụng CNTT, thanh toán không dùng tiền mặt và chuyển đổi số theo lộ trình phù hợp với hoạt động kinh doanh.
+Nguồn: Báo cáo thường niên SaigonBank 2024 · trang PDF 6 (trang in 5)
+Trích đoạn: “Hoàn thành xây dựng Chiến lược phát triển của SAIGONBANK đến năm 2025, định hướng đến năm 2030”
+https://static2.vietstock.vn/data/HNX/2024/BCTN/VN/SGB_Baocaothuongnien_2024/1_sgb_2025_4_17_56f822a_vi_baocaothuongnien_2024.pdf#page=6
+Nguồn: Báo cáo thường niên SaigonBank 2024 · trang PDF 13 (trang in 12)
+Trích đoạn: “Tập trung đẩy mạnh ứng dụng công nghệ thông tin trong hoạt động ngân hàng và hoạt động thanh toán không dùng tiền mặt”
+https://static2.vietstock.vn/data/HNX/2024/BCTN/VN/SGB_Baocaothuongnien_2024/1_sgb_2025_4_17_56f822a_vi_baocaothuongnien_2024.pdf#page=13</v>
       </c>
     </row>
     <row r="44">
@@ -21454,7 +21532,7 @@
         <v>2</v>
       </c>
       <c r="F44" t="s">
-        <v>1390</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="45">
@@ -21474,7 +21552,7 @@
         <v>0</v>
       </c>
       <c r="F45" t="s">
-        <v>1391</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="46">
@@ -21494,10 +21572,10 @@
         <v>3</v>
       </c>
       <c r="F46" t="s">
-        <v>1392</v>
-      </c>
-    </row>
-    <row r="47">
+        <v>1365</v>
+      </c>
+    </row>
+    <row r="47" ht="406" customHeight="1">
       <c r="A47" t="s">
         <v>189</v>
       </c>
@@ -21513,8 +21591,14 @@
       <c r="E47">
         <v>2</v>
       </c>
-      <c r="F47" t="s">
-        <v>1393</v>
+      <c r="F47" s="2" t="str">
+        <v>BCTN 2024 nêu định hướng chuyển đổi số hoạt động kinh doanh theo lộ trình phù hợp cho năm 2025. Báo cáo kết quả năm 2025 ghi nhận nâng cấp SWIFT theo ISO 20022, Oracle 19C, kết nối SIMO và VNeID, phát triển tính năng SAIGONBANK PAY/Smart Banking. Đây là các bước triển khai công nghệ và dịch vụ trong kỳ.
+Nguồn: Báo cáo thường niên SaigonBank 2024 · trang PDF 13 (trang in 12)
+Trích đoạn: “Tập trung đẩy mạnh ứng dụng công nghệ thông tin trong hoạt động ngân hàng và hoạt động thanh toán không dùng tiền mặt”
+https://static2.vietstock.vn/data/HNX/2024/BCTN/VN/SGB_Baocaothuongnien_2024/1_sgb_2025_4_17_56f822a_vi_baocaothuongnien_2024.pdf#page=13
+Nguồn: Báo cáo thường niên SaigonBank 2025 · trang PDF 6 (trang in 5)
+Trích đoạn: “Ngân hàng đã triển khai kết nối tài khoản SAIGONBANK với ứng dụng VNeID của khách hàng liên kết tài khoản SAIGONBANK để nhận chi trả An sinh xã hội qua ứng dụng VNeID”
+https://static2.vietstock.vn/data/HNX/2025/BCTN/VN/SGB_Baocaothuongnien_2025/1_sgb_2026_4_20_43bf2b9_vi_baocaothuongnien_2025_compressedda_ky.pdf#page=6</v>
       </c>
     </row>
     <row r="48">
@@ -21534,7 +21618,7 @@
         <v>2</v>
       </c>
       <c r="F48" t="s">
-        <v>1394</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="49">
@@ -21554,7 +21638,7 @@
         <v>2</v>
       </c>
       <c r="F49" t="s">
-        <v>1395</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="50">
@@ -21574,7 +21658,7 @@
         <v>0</v>
       </c>
       <c r="F50" t="s">
-        <v>1396</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -21594,7 +21678,7 @@
         <v>2</v>
       </c>
       <c r="F51" t="s">
-        <v>1397</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -21614,7 +21698,7 @@
         <v>2</v>
       </c>
       <c r="F52" t="s">
-        <v>1398</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="53" hidden="1">
@@ -21634,7 +21718,7 @@
         <v>2</v>
       </c>
       <c r="F53" t="s">
-        <v>1399</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="54" hidden="1">
@@ -21654,7 +21738,7 @@
         <v>0</v>
       </c>
       <c r="F54" t="s">
-        <v>1400</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="55" hidden="1">
@@ -21674,10 +21758,10 @@
         <v>2</v>
       </c>
       <c r="F55" t="s">
-        <v>1401</v>
-      </c>
-    </row>
-    <row r="56" hidden="1">
+        <v>1373</v>
+      </c>
+    </row>
+    <row r="56" ht="409" hidden="1" customHeight="1">
       <c r="A56" t="s">
         <v>364</v>
       </c>
@@ -21693,8 +21777,17 @@
       <c r="E56">
         <v>2</v>
       </c>
-      <c r="F56" t="s">
-        <v>1402</v>
+      <c r="F56" s="2" t="str">
+        <v>SAIGONBANK ghi nhận hoàn thành xây dựng chiến lược phát triển trong năm 2024 và đặt định hướng ứng dụng CNTT, thanh toán không dùng tiền mặt, chuyển đổi số theo lộ trình cho năm 2025. Báo cáo năm 2025 ghi nhận đầu tư phần cứng, phần mềm, mạng, bảo mật, nâng cấp SWIFT/Oracle và các kết nối dịch vụ theo nhu cầu hoạt động ngân hàng.
+Nguồn: Báo cáo thường niên SaigonBank 2024 · trang PDF 6 (trang in 5)
+Trích đoạn: “Hoàn thành xây dựng Chiến lược phát triển của SAIGONBANK đến năm 2025, định hướng đến năm 2030”
+https://static2.vietstock.vn/data/HNX/2024/BCTN/VN/SGB_Baocaothuongnien_2024/1_sgb_2025_4_17_56f822a_vi_baocaothuongnien_2024.pdf#page=6
+Nguồn: Báo cáo thường niên SaigonBank 2024 · trang PDF 13 (trang in 12)
+Trích đoạn: “Tập trung đẩy mạnh ứng dụng công nghệ thông tin trong hoạt động ngân hàng và hoạt động thanh toán không dùng tiền mặt”
+https://static2.vietstock.vn/data/HNX/2024/BCTN/VN/SGB_Baocaothuongnien_2024/1_sgb_2025_4_17_56f822a_vi_baocaothuongnien_2024.pdf#page=13
+Nguồn: Báo cáo thường niên SaigonBank 2025 · trang PDF 6 (trang in 5)
+Trích đoạn: “Ngân hàng đã triển khai kết nối tài khoản SAIGONBANK với ứng dụng VNeID của khách hàng liên kết tài khoản SAIGONBANK để nhận chi trả An sinh xã hội qua ứng dụng VNeID”
+https://static2.vietstock.vn/data/HNX/2025/BCTN/VN/SGB_Baocaothuongnien_2025/1_sgb_2026_4_20_43bf2b9_vi_baocaothuongnien_2025_compressedda_ky.pdf#page=6</v>
       </c>
     </row>
     <row r="57" hidden="1">
@@ -21714,7 +21807,7 @@
         <v>0</v>
       </c>
       <c r="F57" t="s">
-        <v>1403</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="58" hidden="1">
@@ -21734,7 +21827,7 @@
         <v>0</v>
       </c>
       <c r="F58" t="s">
-        <v>1404</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="59" hidden="1">
@@ -21754,7 +21847,7 @@
         <v>0</v>
       </c>
       <c r="F59" t="s">
-        <v>1405</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="60" hidden="1">
@@ -21774,7 +21867,7 @@
         <v>0</v>
       </c>
       <c r="F60" t="s">
-        <v>1406</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="61" hidden="1">
@@ -21794,7 +21887,7 @@
         <v>0</v>
       </c>
       <c r="F61" t="s">
-        <v>1407</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="62" hidden="1">
@@ -21814,7 +21907,7 @@
         <v>2</v>
       </c>
       <c r="F62" t="s">
-        <v>1408</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="63" hidden="1">
@@ -21834,7 +21927,7 @@
         <v>0</v>
       </c>
       <c r="F63" t="s">
-        <v>1409</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="64" hidden="1">
@@ -21854,7 +21947,7 @@
         <v>2</v>
       </c>
       <c r="F64" t="s">
-        <v>1410</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="65" hidden="1">
@@ -21874,7 +21967,7 @@
         <v>3</v>
       </c>
       <c r="F65" t="s">
-        <v>1411</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="66" hidden="1">
@@ -21894,7 +21987,7 @@
         <v>0</v>
       </c>
       <c r="F66" t="s">
-        <v>1412</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="67" hidden="1">
@@ -21914,7 +22007,7 @@
         <v>2</v>
       </c>
       <c r="F67" t="s">
-        <v>1413</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="68" hidden="1">
@@ -21934,7 +22027,7 @@
         <v>0</v>
       </c>
       <c r="F68" t="s">
-        <v>1414</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="69" hidden="1">
@@ -21954,7 +22047,7 @@
         <v>0</v>
       </c>
       <c r="F69" t="s">
-        <v>1415</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="70" hidden="1">
@@ -21974,7 +22067,7 @@
         <v>0</v>
       </c>
       <c r="F70" t="s">
-        <v>1416</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="71" hidden="1">
@@ -21994,7 +22087,7 @@
         <v>0</v>
       </c>
       <c r="F71" t="s">
-        <v>1417</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="72" hidden="1">
@@ -22014,7 +22107,7 @@
         <v>2</v>
       </c>
       <c r="F72" t="s">
-        <v>1418</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="73" hidden="1">
@@ -22034,7 +22127,7 @@
         <v>0</v>
       </c>
       <c r="F73" t="s">
-        <v>1419</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="74" hidden="1">
@@ -22054,7 +22147,7 @@
         <v>0</v>
       </c>
       <c r="F74" t="s">
-        <v>1420</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="75" hidden="1">
@@ -22074,7 +22167,7 @@
         <v>2</v>
       </c>
       <c r="F75" t="s">
-        <v>1421</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="76" hidden="1">
@@ -22094,7 +22187,7 @@
         <v>0</v>
       </c>
       <c r="F76" t="s">
-        <v>1422</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="77" hidden="1">
@@ -22114,7 +22207,7 @@
         <v>0</v>
       </c>
       <c r="F77" t="s">
-        <v>1423</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="78" hidden="1">
@@ -22134,7 +22227,7 @@
         <v>0</v>
       </c>
       <c r="F78" t="s">
-        <v>1424</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="79" hidden="1">
@@ -22154,7 +22247,7 @@
         <v>2</v>
       </c>
       <c r="F79" t="s">
-        <v>1425</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="80" hidden="1">
@@ -22174,7 +22267,7 @@
         <v>2</v>
       </c>
       <c r="F80" t="s">
-        <v>1426</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="81" hidden="1">
@@ -22194,7 +22287,7 @@
         <v>3</v>
       </c>
       <c r="F81" t="s">
-        <v>1427</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="82" hidden="1">
@@ -22214,7 +22307,7 @@
         <v>3</v>
       </c>
       <c r="F82" t="s">
-        <v>1428</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="83" hidden="1">
@@ -22234,7 +22327,7 @@
         <v>0</v>
       </c>
       <c r="F83" t="s">
-        <v>1429</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="84" hidden="1">
@@ -22254,7 +22347,7 @@
         <v>2</v>
       </c>
       <c r="F84" t="s">
-        <v>1430</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="85" hidden="1">
@@ -22274,7 +22367,7 @@
         <v>0</v>
       </c>
       <c r="F85" t="s">
-        <v>1431</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="86" hidden="1">
@@ -22294,7 +22387,7 @@
         <v>0</v>
       </c>
       <c r="F86" t="s">
-        <v>1432</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="87" hidden="1">
@@ -22314,7 +22407,7 @@
         <v>2</v>
       </c>
       <c r="F87" t="s">
-        <v>1433</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="88" hidden="1">
@@ -22334,7 +22427,7 @@
         <v>2</v>
       </c>
       <c r="F88" t="s">
-        <v>1434</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="89" hidden="1">
@@ -22354,7 +22447,7 @@
         <v>2</v>
       </c>
       <c r="F89" t="s">
-        <v>1435</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="90" hidden="1">
@@ -22374,7 +22467,7 @@
         <v>2</v>
       </c>
       <c r="F90" t="s">
-        <v>1436</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="91" hidden="1">
@@ -22394,7 +22487,7 @@
         <v>0</v>
       </c>
       <c r="F91" t="s">
-        <v>1437</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="92" hidden="1">
@@ -22414,7 +22507,7 @@
         <v>0</v>
       </c>
       <c r="F92" t="s">
-        <v>1438</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="93" hidden="1">
@@ -22434,7 +22527,7 @@
         <v>0</v>
       </c>
       <c r="F93" t="s">
-        <v>1439</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="94" hidden="1">
@@ -22454,7 +22547,7 @@
         <v>2</v>
       </c>
       <c r="F94" t="s">
-        <v>1440</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="95" hidden="1">
@@ -22474,7 +22567,7 @@
         <v>0</v>
       </c>
       <c r="F95" t="s">
-        <v>1441</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="96" hidden="1">
@@ -22494,7 +22587,7 @@
         <v>0</v>
       </c>
       <c r="F96" t="s">
-        <v>1442</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="97" hidden="1">
@@ -22514,7 +22607,7 @@
         <v>2</v>
       </c>
       <c r="F97" t="s">
-        <v>1443</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="98" hidden="1">
@@ -22534,7 +22627,7 @@
         <v>2</v>
       </c>
       <c r="F98" t="s">
-        <v>1444</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="99" hidden="1">
@@ -22554,7 +22647,7 @@
         <v>0</v>
       </c>
       <c r="F99" t="s">
-        <v>1445</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="100" hidden="1">
@@ -22574,7 +22667,7 @@
         <v>2</v>
       </c>
       <c r="F100" t="s">
-        <v>1446</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="101" hidden="1">
@@ -22594,7 +22687,7 @@
         <v>2</v>
       </c>
       <c r="F101" t="s">
-        <v>1447</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="102" hidden="1">
@@ -22614,7 +22707,7 @@
         <v>2</v>
       </c>
       <c r="F102" t="s">
-        <v>1448</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="103" hidden="1">
@@ -22634,7 +22727,7 @@
         <v>2</v>
       </c>
       <c r="F103" t="s">
-        <v>1449</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="104" hidden="1">
@@ -22654,7 +22747,7 @@
         <v>0</v>
       </c>
       <c r="F104" t="s">
-        <v>1450</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="105" hidden="1">
@@ -22674,7 +22767,7 @@
         <v>0</v>
       </c>
       <c r="F105" t="s">
-        <v>1451</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="106" hidden="1">
@@ -22694,7 +22787,7 @@
         <v>2</v>
       </c>
       <c r="F106" t="s">
-        <v>1452</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="107" hidden="1">
@@ -22714,7 +22807,7 @@
         <v>0</v>
       </c>
       <c r="F107" t="s">
-        <v>1453</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="108" hidden="1">
@@ -22734,7 +22827,7 @@
         <v>0</v>
       </c>
       <c r="F108" t="s">
-        <v>1454</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="109" hidden="1">
@@ -22754,7 +22847,7 @@
         <v>2</v>
       </c>
       <c r="F109" t="s">
-        <v>1455</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="110" hidden="1">
@@ -22774,7 +22867,7 @@
         <v>0</v>
       </c>
       <c r="F110" t="s">
-        <v>1456</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="111" hidden="1">
@@ -22794,7 +22887,7 @@
         <v>0</v>
       </c>
       <c r="F111" t="s">
-        <v>1457</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="112" hidden="1">
@@ -22814,7 +22907,7 @@
         <v>2</v>
       </c>
       <c r="F112" t="s">
-        <v>1458</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="113" hidden="1">
@@ -22834,7 +22927,7 @@
         <v>2</v>
       </c>
       <c r="F113" t="s">
-        <v>1459</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="114" hidden="1">
@@ -22854,7 +22947,7 @@
         <v>0</v>
       </c>
       <c r="F114" t="s">
-        <v>1460</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="115" hidden="1">
@@ -22874,7 +22967,7 @@
         <v>0</v>
       </c>
       <c r="F115" t="s">
-        <v>1461</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="116" hidden="1">
@@ -22894,7 +22987,7 @@
         <v>2</v>
       </c>
       <c r="F116" t="s">
-        <v>1462</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="117" hidden="1">
@@ -22914,7 +23007,7 @@
         <v>0</v>
       </c>
       <c r="F117" t="s">
-        <v>1463</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="118" hidden="1">
@@ -22934,7 +23027,7 @@
         <v>2</v>
       </c>
       <c r="F118" t="s">
-        <v>1464</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="119" hidden="1">
@@ -22954,7 +23047,7 @@
         <v>0</v>
       </c>
       <c r="F119" t="s">
-        <v>1465</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="120" hidden="1">
@@ -22974,7 +23067,7 @@
         <v>2</v>
       </c>
       <c r="F120" t="s">
-        <v>1466</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="121" hidden="1">
@@ -22994,7 +23087,7 @@
         <v>0</v>
       </c>
       <c r="F121" t="s">
-        <v>1467</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="122" hidden="1">
@@ -23014,7 +23107,7 @@
         <v>0</v>
       </c>
       <c r="F122" t="s">
-        <v>1468</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="123" hidden="1">
@@ -23034,7 +23127,7 @@
         <v>2</v>
       </c>
       <c r="F123" t="s">
-        <v>1469</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="124" hidden="1">
@@ -23054,7 +23147,7 @@
         <v>0</v>
       </c>
       <c r="F124" t="s">
-        <v>1470</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="125" hidden="1">
@@ -23074,7 +23167,7 @@
         <v>0</v>
       </c>
       <c r="F125" t="s">
-        <v>1471</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="126" hidden="1">
@@ -23094,7 +23187,7 @@
         <v>0</v>
       </c>
       <c r="F126" t="s">
-        <v>1472</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="127" hidden="1">
@@ -23114,7 +23207,7 @@
         <v>3</v>
       </c>
       <c r="F127" t="s">
-        <v>1473</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="128" hidden="1">
@@ -23134,7 +23227,7 @@
         <v>2</v>
       </c>
       <c r="F128" t="s">
-        <v>1474</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="129" hidden="1">
@@ -23154,7 +23247,7 @@
         <v>0</v>
       </c>
       <c r="F129" t="s">
-        <v>1475</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="130" hidden="1">
@@ -23174,7 +23267,7 @@
         <v>0</v>
       </c>
       <c r="F130" t="s">
-        <v>1476</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="131" hidden="1">
@@ -23216,7 +23309,7 @@
         <v>0</v>
       </c>
       <c r="F132" t="s">
-        <v>1477</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="133" hidden="1">
@@ -23236,7 +23329,7 @@
         <v>0</v>
       </c>
       <c r="F133" t="s">
-        <v>1478</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="134" hidden="1">
@@ -23256,7 +23349,7 @@
         <v>0</v>
       </c>
       <c r="F134" t="s">
-        <v>1479</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="135" hidden="1">
@@ -23276,7 +23369,7 @@
         <v>0</v>
       </c>
       <c r="F135" t="s">
-        <v>1480</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="136" hidden="1">
@@ -23296,7 +23389,7 @@
         <v>2</v>
       </c>
       <c r="F136" t="s">
-        <v>1481</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="137" hidden="1">
@@ -23316,7 +23409,7 @@
         <v>0</v>
       </c>
       <c r="F137" t="s">
-        <v>1482</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="138" hidden="1">
@@ -23336,7 +23429,7 @@
         <v>0</v>
       </c>
       <c r="F138" t="s">
-        <v>1483</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="139" hidden="1">
@@ -23356,7 +23449,7 @@
         <v>2</v>
       </c>
       <c r="F139" t="s">
-        <v>1484</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="140" hidden="1">
@@ -23376,7 +23469,7 @@
         <v>2</v>
       </c>
       <c r="F140" t="s">
-        <v>1485</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="141" hidden="1">
@@ -23396,7 +23489,7 @@
         <v>0</v>
       </c>
       <c r="F141" t="s">
-        <v>1486</v>
+        <v>1457</v>
       </c>
     </row>
   </sheetData>
@@ -23426,30 +23519,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1487</v>
+        <v>1458</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1488</v>
+        <v>1459</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1489</v>
+        <v>1460</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1490</v>
+        <v>1461</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1491</v>
+        <v>1462</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1492</v>
+        <v>1463</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1493</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1494</v>
+        <v>1465</v>
       </c>
       <c r="B2">
         <v>140</v>
@@ -23472,7 +23565,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1495</v>
+        <v>1466</v>
       </c>
       <c r="B3">
         <v>140</v>
@@ -23495,7 +23588,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1496</v>
+        <v>1467</v>
       </c>
       <c r="B4">
         <v>140</v>
@@ -23518,7 +23611,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1497</v>
+        <v>1468</v>
       </c>
       <c r="B5">
         <v>140</v>
@@ -23541,7 +23634,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1498</v>
+        <v>1469</v>
       </c>
       <c r="B6">
         <v>140</v>

</xml_diff>

<commit_message>
Make revised evidence citations readable in final Excel workbooks
</commit_message>
<xml_diff>
--- a/Code/CleanData.xlsx
+++ b/Code/CleanData.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh_muc" sheetId="1" r:id="R7736cafa2a104168"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TPBank" sheetId="2" r:id="R52b126d43a9c4add"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDBank" sheetId="3" r:id="Re15cde1358304955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LP Bank" sheetId="4" r:id="R846d4f46dcc74373"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OCB" sheetId="5" r:id="R08646ca547c9445c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SaigonBank" sheetId="6" r:id="Rb61bc0d15e1644c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong_hop" sheetId="7" r:id="R3f4cf67300424cc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh_muc" sheetId="1" r:id="R33391d88e5ca405e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TPBank" sheetId="2" r:id="R4a4a44acaa75426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HDBank" sheetId="3" r:id="R97370eb3e73545b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LP Bank" sheetId="4" r:id="R1d06afbcb9e64cc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OCB" sheetId="5" r:id="Rd189871b351944ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SaigonBank" sheetId="6" r:id="R0cb96016a1604cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong_hop" sheetId="7" r:id="Rf8d565c144ac4dce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14780,7 +14780,7 @@
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="55" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="55" customWidth="1"/>
+    <col min="6" max="6" width="110" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14803,7 +14803,7 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="2" ht="336" hidden="1" customHeight="1">
+    <row r="2" ht="182" hidden="1" customHeight="1">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -14849,7 +14849,7 @@
         <v>1115</v>
       </c>
     </row>
-    <row r="4" ht="196" hidden="1" customHeight="1">
+    <row r="4" ht="112" hidden="1" customHeight="1">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -15012,7 +15012,7 @@
         <v>1121</v>
       </c>
     </row>
-    <row r="12" ht="336" hidden="1" customHeight="1">
+    <row r="12" ht="182" hidden="1" customHeight="1">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -15038,7 +15038,7 @@
 https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=26</v>
       </c>
     </row>
-    <row r="13" ht="336" hidden="1" customHeight="1">
+    <row r="13" ht="182" hidden="1" customHeight="1">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -15064,7 +15064,7 @@
 https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=32</v>
       </c>
     </row>
-    <row r="14" ht="409" hidden="1" customHeight="1">
+    <row r="14" ht="252" hidden="1" customHeight="1">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -15213,7 +15213,7 @@
         <v>1127</v>
       </c>
     </row>
-    <row r="21" ht="350" hidden="1" customHeight="1">
+    <row r="21" ht="182" hidden="1" customHeight="1">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -15299,7 +15299,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="25" ht="350" hidden="1" customHeight="1">
+    <row r="25" ht="182" hidden="1" customHeight="1">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -15445,7 +15445,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="32" ht="350" hidden="1" customHeight="1">
+    <row r="32" ht="182" hidden="1" customHeight="1">
       <c r="A32" t="s">
         <v>189</v>
       </c>
@@ -15531,7 +15531,7 @@
         <v>1135</v>
       </c>
     </row>
-    <row r="36" ht="350" hidden="1" customHeight="1">
+    <row r="36" ht="182" hidden="1" customHeight="1">
       <c r="A36" t="s">
         <v>189</v>
       </c>
@@ -15617,7 +15617,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="40" ht="336" hidden="1" customHeight="1">
+    <row r="40" ht="182" hidden="1" customHeight="1">
       <c r="A40" t="s">
         <v>189</v>
       </c>
@@ -15643,7 +15643,7 @@
 https://static2.vietstock.vn/data/HOSE/2024/BCTN/VN/LPB_Baocaothuongnien_2024.pdf#page=32</v>
       </c>
     </row>
-    <row r="41" ht="336" hidden="1" customHeight="1">
+    <row r="41" ht="182" hidden="1" customHeight="1">
       <c r="A41" t="s">
         <v>189</v>
       </c>
@@ -15669,7 +15669,7 @@
 https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=27</v>
       </c>
     </row>
-    <row r="42" ht="364" hidden="1" customHeight="1">
+    <row r="42" ht="196" hidden="1" customHeight="1">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -15935,7 +15935,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="55" ht="364" hidden="1" customHeight="1">
+    <row r="55" ht="196" hidden="1" customHeight="1">
       <c r="A55" t="s">
         <v>364</v>
       </c>
@@ -16021,7 +16021,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="59" ht="350" hidden="1" customHeight="1">
+    <row r="59" ht="182" hidden="1" customHeight="1">
       <c r="A59" t="s">
         <v>364</v>
       </c>
@@ -16127,7 +16127,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="64" ht="238" hidden="1" customHeight="1">
+    <row r="64" ht="126" hidden="1" customHeight="1">
       <c r="A64" t="s">
         <v>364</v>
       </c>
@@ -16190,7 +16190,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="67" ht="364" hidden="1" customHeight="1">
+    <row r="67" ht="182" hidden="1" customHeight="1">
       <c r="A67" t="s">
         <v>364</v>
       </c>
@@ -16396,7 +16396,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="77" ht="364" hidden="1" customHeight="1">
+    <row r="77" ht="182" hidden="1" customHeight="1">
       <c r="A77" t="s">
         <v>364</v>
       </c>
@@ -16562,7 +16562,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="85" ht="336" hidden="1" customHeight="1">
+    <row r="85" ht="182" hidden="1" customHeight="1">
       <c r="A85" t="s">
         <v>573</v>
       </c>
@@ -16628,7 +16628,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="88" ht="409" hidden="1" customHeight="1">
+    <row r="88" ht="252" hidden="1" customHeight="1">
       <c r="A88" t="s">
         <v>573</v>
       </c>
@@ -16697,7 +16697,7 @@
         <v>1171</v>
       </c>
     </row>
-    <row r="91" ht="350" hidden="1" customHeight="1">
+    <row r="91" ht="182" hidden="1" customHeight="1">
       <c r="A91" t="s">
         <v>573</v>
       </c>
@@ -16883,7 +16883,7 @@
         <v>1175</v>
       </c>
     </row>
-    <row r="100" ht="409" hidden="1" customHeight="1">
+    <row r="100" ht="266" hidden="1" customHeight="1">
       <c r="A100" t="s">
         <v>573</v>
       </c>
@@ -16912,7 +16912,7 @@
 https://static2.vietstock.vn/data/HOSE/2025/BCTN/VN/LPB_Baocaothuongnien_2025.pdf#page=36</v>
       </c>
     </row>
-    <row r="101" ht="364" hidden="1" customHeight="1">
+    <row r="101" ht="196" hidden="1" customHeight="1">
       <c r="A101" t="s">
         <v>573</v>
       </c>
@@ -17438,7 +17438,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="127" ht="364" customHeight="1">
+    <row r="127" ht="182" customHeight="1">
       <c r="A127" t="s">
         <v>890</v>
       </c>
@@ -17704,7 +17704,7 @@
         <v>1193</v>
       </c>
     </row>
-    <row r="140" ht="378" customHeight="1">
+    <row r="140" ht="196" customHeight="1">
       <c r="A140" t="s">
         <v>890</v>
       </c>
@@ -20637,7 +20637,7 @@
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="55" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="55" customWidth="1"/>
+    <col min="6" max="6" width="110" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21260,7 +21260,7 @@
         <v>1353</v>
       </c>
     </row>
-    <row r="32" ht="280" customHeight="1">
+    <row r="32" ht="140" customHeight="1">
       <c r="A32" t="s">
         <v>189</v>
       </c>
@@ -21443,7 +21443,7 @@
         <v>1361</v>
       </c>
     </row>
-    <row r="41" ht="406" customHeight="1">
+    <row r="41" ht="224" customHeight="1">
       <c r="A41" t="s">
         <v>189</v>
       </c>
@@ -21489,7 +21489,7 @@
         <v>1362</v>
       </c>
     </row>
-    <row r="43" ht="378" customHeight="1">
+    <row r="43" ht="224" customHeight="1">
       <c r="A43" t="s">
         <v>189</v>
       </c>
@@ -21575,7 +21575,7 @@
         <v>1365</v>
       </c>
     </row>
-    <row r="47" ht="406" customHeight="1">
+    <row r="47" ht="224" customHeight="1">
       <c r="A47" t="s">
         <v>189</v>
       </c>
@@ -21761,7 +21761,7 @@
         <v>1373</v>
       </c>
     </row>
-    <row r="56" ht="409" hidden="1" customHeight="1">
+    <row r="56" ht="308" hidden="1" customHeight="1">
       <c r="A56" t="s">
         <v>364</v>
       </c>

</xml_diff>

<commit_message>
Correct LPBank pillar heading in final CleanData workbook
</commit_message>
<xml_diff>
--- a/Code/CleanData.xlsx
+++ b/Code/CleanData.xlsx
@@ -14784,8 +14784,8 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>1114</v>
+      <c r="A1" s="1" t="str">
+        <v>Trụ cột</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>

</xml_diff>